<commit_message>
Add guided pay package examples and ignore sample rows
</commit_message>
<xml_diff>
--- a/public/templates/Pay-Packages-Batch-Template.xlsx
+++ b/public/templates/Pay-Packages-Batch-Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rb3704a1b5a1449c6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="R5a1f18d16f40480d"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R469035307d13433e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R51a28096f1b24144"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="R5699423ccae94e05"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R3e16e1c8c64048cf"/>
   </sheets>
 </workbook>
 </file>
@@ -20,7 +20,7 @@
     <numFmt numFmtId="201" formatCode="#,##0.00"/>
     <numFmt numFmtId="202" formatCode="@"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -31,18 +31,29 @@
       <name val="Carlito"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF92400E"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -56,19 +67,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="200" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="201" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="202" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -278,10 +296,10 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="7" t="str">
+      <c r="A1" s="14" t="str">
         <v>PAY PACKAGES · BATCH UPLOAD</v>
       </c>
-      <c r="B1" s="7" t="str">
+      <c r="B1" s="14" t="str">
         <v>Instructions</v>
       </c>
     </row>
@@ -391,33 +409,49 @@
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="1" t="str">
-        <v>14. Review</v>
+        <v>14. Examples</v>
       </c>
       <c r="B15" s="1" t="str">
-        <v>Tax, contribution, proration and 13th-month treatments remain unreviewed. HR must review and authorize drafts.</v>
+        <v>Rows whose Package key begins with EXAMPLE- are included for guidance and ignored automatically during upload. Delete them if you prefer a blank sheet.</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="1" t="str">
-        <v>15. Existing dates</v>
+        <v>15. Dual arrangements</v>
       </c>
       <c r="B16" s="1" t="str">
-        <v>Imports reject existing non-rejected packages for the same employee, engagement and effective date. Use the individual form for corrections.</v>
+        <v>Use the same Employee code on two rows: one employee_payroll row and one professional_fee row with a distinct Engagement reference.</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="1" t="str">
-        <v>16. Interrupted save</v>
+        <v>16. Review</v>
       </c>
       <c r="B17" s="1" t="str">
-        <v>Saving stops at the first failure. Earlier drafts remain saved. Check existing drafts before uploading only remaining rows.</v>
+        <v>Tax, contribution, proration and 13th-month treatments remain unreviewed. HR must review and authorize drafts.</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="1" t="str">
+        <v>17. Existing dates</v>
+      </c>
+      <c r="B18" s="1" t="str">
+        <v>Imports reject existing non-rejected packages for the same employee, engagement and effective date. Use the individual form for corrections.</v>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="1" t="str">
+        <v>18. Interrupted save</v>
+      </c>
+      <c r="B19" s="1" t="str">
+        <v>Saving stops at the first failure. Earlier drafts remain saved. Check existing drafts before uploading only remaining rows.</v>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="1" t="str">
         <v>Available BU names</v>
       </c>
-      <c r="B18" s="1" t="str">
+      <c r="B20" s="1" t="str">
         <v>The Fun Roof; The Dessert Museum; Gootopia SM North Edsa; Bakebe - S Maison; Bakebe - SM Aura; Gootopia - SM MOA; Inflatable Island Beach Club; TNG (Corporation)</v>
       </c>
     </row>
@@ -445,107 +479,187 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="7" t="str">
+      <c r="A1" s="14" t="str">
         <v>Package key</v>
       </c>
-      <c r="B1" s="7" t="str">
+      <c r="B1" s="14" t="str">
         <v>Employee code</v>
       </c>
-      <c r="C1" s="7" t="str">
+      <c r="C1" s="14" t="str">
         <v>Business unit / payroll group</v>
       </c>
-      <c r="D1" s="7" t="str">
+      <c r="D1" s="14" t="str">
         <v>Pay stream</v>
       </c>
-      <c r="E1" s="7" t="str">
+      <c r="E1" s="14" t="str">
         <v>Effective from</v>
       </c>
-      <c r="F1" s="7" t="str">
+      <c r="F1" s="14" t="str">
         <v>Amount unit</v>
       </c>
-      <c r="G1" s="7" t="str">
+      <c r="G1" s="14" t="str">
         <v>Basic pay / fee amount</v>
       </c>
-      <c r="H1" s="7" t="str">
+      <c r="H1" s="14" t="str">
         <v>PAN ID (optional)</v>
       </c>
-      <c r="I1" s="7" t="str">
+      <c r="I1" s="14" t="str">
         <v>Source reference</v>
       </c>
-      <c r="J1" s="7" t="str">
+      <c r="J1" s="14" t="str">
         <v>Reason</v>
       </c>
-      <c r="K1" s="7" t="str">
+      <c r="K1" s="14" t="str">
         <v>Engagement reference</v>
       </c>
-      <c r="L1" s="7" t="str">
+      <c r="L1" s="14" t="str">
         <v>Tax profile reference</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
+      <c r="A2" s="9" t="str">
+        <v>EXAMPLE-EMP-001</v>
+      </c>
+      <c r="B2" s="9" t="str">
+        <v>TNG-EXAMPLE-001</v>
+      </c>
+      <c r="C2" s="9" t="str">
+        <v>The Fun Roof</v>
+      </c>
+      <c r="D2" s="9" t="str">
+        <v>employee_payroll</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F2" s="4" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H2" s="4" t="str"/>
+      <c r="I2" s="4" t="str">
+        <v>Current HRIS record</v>
+      </c>
+      <c r="J2" s="4" t="str">
+        <v>Example only — replace with approved source</v>
+      </c>
+      <c r="K2" s="4" t="str"/>
+      <c r="L2" s="4" t="str"/>
     </row>
     <row r="3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
+      <c r="A3" s="9" t="str">
+        <v>EXAMPLE-CONS-001</v>
+      </c>
+      <c r="B3" s="9" t="str">
+        <v>TNG-EXAMPLE-002</v>
+      </c>
+      <c r="C3" s="9" t="str">
+        <v>TNG (Corporation)</v>
+      </c>
+      <c r="D3" s="9" t="str">
+        <v>professional_fee</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F3" s="4" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>45000</v>
+      </c>
+      <c r="H3" s="4" t="str"/>
+      <c r="I3" s="4" t="str">
+        <v>Approved consultant agreement</v>
+      </c>
+      <c r="J3" s="4" t="str">
+        <v>Example only — replace with approved agreement</v>
+      </c>
+      <c r="K3" s="4" t="str">
+        <v>CONSULTING-2026-001</v>
+      </c>
+      <c r="L3" s="4" t="str">
+        <v>TAX-PROFILE-2026-001</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="A4" s="9" t="str">
+        <v>EXAMPLE-DUAL-EMP</v>
+      </c>
+      <c r="B4" s="9" t="str">
+        <v>TNG-EXAMPLE-003</v>
+      </c>
+      <c r="C4" s="9" t="str">
+        <v>The Fun Roof</v>
+      </c>
+      <c r="D4" s="9" t="str">
+        <v>employee_payroll</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F4" s="4" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H4" s="4" t="str"/>
+      <c r="I4" s="4" t="str">
+        <v>Current HRIS record</v>
+      </c>
+      <c r="J4" s="4" t="str">
+        <v>Example employment side of dual arrangement</v>
+      </c>
+      <c r="K4" s="4" t="str"/>
+      <c r="L4" s="4" t="str"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
+      <c r="A5" s="9" t="str">
+        <v>EXAMPLE-DUAL-CONS</v>
+      </c>
+      <c r="B5" s="9" t="str">
+        <v>TNG-EXAMPLE-003</v>
+      </c>
+      <c r="C5" s="9" t="str">
+        <v>TNG (Corporation)</v>
+      </c>
+      <c r="D5" s="9" t="str">
+        <v>professional_fee</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F5" s="4" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H5" s="4" t="str"/>
+      <c r="I5" s="4" t="str">
+        <v>Approved consultant agreement</v>
+      </c>
+      <c r="J5" s="4" t="str">
+        <v>Example consultant side of dual arrangement</v>
+      </c>
+      <c r="K5" s="4" t="str">
+        <v>CONSULTING-2026-003</v>
+      </c>
+      <c r="L5" s="4" t="str">
+        <v>TAX-PROFILE-2026-003</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="3"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="7"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="4"/>
+      <c r="G6" s="8"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -553,13 +667,13 @@
       <c r="L6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="3"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="4"/>
+      <c r="G7" s="8"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -567,13 +681,13 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="3"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="4"/>
+      <c r="G8" s="8"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -581,13 +695,13 @@
       <c r="L8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="3"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="7"/>
       <c r="F9" s="2"/>
-      <c r="G9" s="4"/>
+      <c r="G9" s="8"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -595,13 +709,13 @@
       <c r="L9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="3"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="7"/>
       <c r="F10" s="2"/>
-      <c r="G10" s="4"/>
+      <c r="G10" s="8"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -609,13 +723,13 @@
       <c r="L10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="3"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="7"/>
       <c r="F11" s="2"/>
-      <c r="G11" s="4"/>
+      <c r="G11" s="8"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -623,13 +737,13 @@
       <c r="L11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="3"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="4"/>
+      <c r="G12" s="8"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -637,13 +751,13 @@
       <c r="L12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="3"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="2"/>
-      <c r="G13" s="4"/>
+      <c r="G13" s="8"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -651,13 +765,13 @@
       <c r="L13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="3"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="7"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="4"/>
+      <c r="G14" s="8"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -665,13 +779,13 @@
       <c r="L14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="3"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="7"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="4"/>
+      <c r="G15" s="8"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -679,13 +793,13 @@
       <c r="L15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="3"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="4"/>
+      <c r="G16" s="8"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -693,13 +807,13 @@
       <c r="L16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="3"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="4"/>
+      <c r="G17" s="8"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -707,13 +821,13 @@
       <c r="L17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="3"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="4"/>
+      <c r="G18" s="8"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -721,13 +835,13 @@
       <c r="L18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="3"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="4"/>
+      <c r="G19" s="8"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -735,13 +849,13 @@
       <c r="L19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="3"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="4"/>
+      <c r="G20" s="8"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -749,13 +863,13 @@
       <c r="L20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="3"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="4"/>
+      <c r="G21" s="8"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -763,13 +877,13 @@
       <c r="L21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="3"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="7"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="4"/>
+      <c r="G22" s="8"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -777,13 +891,13 @@
       <c r="L22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="3"/>
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="7"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="4"/>
+      <c r="G23" s="8"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -791,13 +905,13 @@
       <c r="L23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="3"/>
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="2"/>
-      <c r="G24" s="4"/>
+      <c r="G24" s="8"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
@@ -805,13 +919,13 @@
       <c r="L24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="3"/>
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="2"/>
-      <c r="G25" s="4"/>
+      <c r="G25" s="8"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
@@ -819,13 +933,13 @@
       <c r="L25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="3"/>
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="2"/>
-      <c r="G26" s="4"/>
+      <c r="G26" s="8"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
@@ -833,13 +947,13 @@
       <c r="L26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="3"/>
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="2"/>
-      <c r="G27" s="4"/>
+      <c r="G27" s="8"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
@@ -847,13 +961,13 @@
       <c r="L27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="3"/>
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="2"/>
-      <c r="G28" s="4"/>
+      <c r="G28" s="8"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
@@ -861,13 +975,13 @@
       <c r="L28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="3"/>
+      <c r="A29" s="10"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="7"/>
       <c r="F29" s="2"/>
-      <c r="G29" s="4"/>
+      <c r="G29" s="8"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -875,13 +989,13 @@
       <c r="L29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="3"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="2"/>
-      <c r="G30" s="4"/>
+      <c r="G30" s="8"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -889,13 +1003,13 @@
       <c r="L30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="3"/>
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="7"/>
       <c r="F31" s="2"/>
-      <c r="G31" s="4"/>
+      <c r="G31" s="8"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
@@ -903,13 +1017,13 @@
       <c r="L31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="3"/>
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="7"/>
       <c r="F32" s="2"/>
-      <c r="G32" s="4"/>
+      <c r="G32" s="8"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -917,13 +1031,13 @@
       <c r="L32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="3"/>
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="7"/>
       <c r="F33" s="2"/>
-      <c r="G33" s="4"/>
+      <c r="G33" s="8"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -931,13 +1045,13 @@
       <c r="L33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="3"/>
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="7"/>
       <c r="F34" s="2"/>
-      <c r="G34" s="4"/>
+      <c r="G34" s="8"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -945,13 +1059,13 @@
       <c r="L34" s="2"/>
     </row>
     <row r="35">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="3"/>
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="7"/>
       <c r="F35" s="2"/>
-      <c r="G35" s="4"/>
+      <c r="G35" s="8"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -959,13 +1073,13 @@
       <c r="L35" s="2"/>
     </row>
     <row r="36">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="3"/>
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="2"/>
-      <c r="G36" s="4"/>
+      <c r="G36" s="8"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -973,13 +1087,13 @@
       <c r="L36" s="2"/>
     </row>
     <row r="37">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="3"/>
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="7"/>
       <c r="F37" s="2"/>
-      <c r="G37" s="4"/>
+      <c r="G37" s="8"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -987,13 +1101,13 @@
       <c r="L37" s="2"/>
     </row>
     <row r="38">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="3"/>
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="7"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="4"/>
+      <c r="G38" s="8"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -1001,13 +1115,13 @@
       <c r="L38" s="2"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="3"/>
+      <c r="A39" s="10"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="2"/>
-      <c r="G39" s="4"/>
+      <c r="G39" s="8"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -1015,13 +1129,13 @@
       <c r="L39" s="2"/>
     </row>
     <row r="40">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="3"/>
+      <c r="A40" s="10"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="7"/>
       <c r="F40" s="2"/>
-      <c r="G40" s="4"/>
+      <c r="G40" s="8"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
@@ -1029,13 +1143,13 @@
       <c r="L40" s="2"/>
     </row>
     <row r="41">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="3"/>
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="7"/>
       <c r="F41" s="2"/>
-      <c r="G41" s="4"/>
+      <c r="G41" s="8"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
@@ -1043,13 +1157,13 @@
       <c r="L41" s="2"/>
     </row>
     <row r="42">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="3"/>
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="7"/>
       <c r="F42" s="2"/>
-      <c r="G42" s="4"/>
+      <c r="G42" s="8"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
@@ -1057,13 +1171,13 @@
       <c r="L42" s="2"/>
     </row>
     <row r="43">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="3"/>
+      <c r="A43" s="10"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="7"/>
       <c r="F43" s="2"/>
-      <c r="G43" s="4"/>
+      <c r="G43" s="8"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
@@ -1071,13 +1185,13 @@
       <c r="L43" s="2"/>
     </row>
     <row r="44">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="3"/>
+      <c r="A44" s="10"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="2"/>
-      <c r="G44" s="4"/>
+      <c r="G44" s="8"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
@@ -1085,13 +1199,13 @@
       <c r="L44" s="2"/>
     </row>
     <row r="45">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="3"/>
+      <c r="A45" s="10"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="7"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="4"/>
+      <c r="G45" s="8"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
@@ -1099,13 +1213,13 @@
       <c r="L45" s="2"/>
     </row>
     <row r="46">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="3"/>
+      <c r="A46" s="10"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="7"/>
       <c r="F46" s="2"/>
-      <c r="G46" s="4"/>
+      <c r="G46" s="8"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
@@ -1113,13 +1227,13 @@
       <c r="L46" s="2"/>
     </row>
     <row r="47">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="3"/>
+      <c r="A47" s="10"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="4"/>
+      <c r="G47" s="8"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
@@ -1127,13 +1241,13 @@
       <c r="L47" s="2"/>
     </row>
     <row r="48">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="3"/>
+      <c r="A48" s="10"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="2"/>
-      <c r="G48" s="4"/>
+      <c r="G48" s="8"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
@@ -1141,13 +1255,13 @@
       <c r="L48" s="2"/>
     </row>
     <row r="49">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="3"/>
+      <c r="A49" s="10"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="7"/>
       <c r="F49" s="2"/>
-      <c r="G49" s="4"/>
+      <c r="G49" s="8"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
@@ -1155,13 +1269,13 @@
       <c r="L49" s="2"/>
     </row>
     <row r="50">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="3"/>
+      <c r="A50" s="10"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="7"/>
       <c r="F50" s="2"/>
-      <c r="G50" s="4"/>
+      <c r="G50" s="8"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
@@ -1169,13 +1283,13 @@
       <c r="L50" s="2"/>
     </row>
     <row r="51">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="3"/>
+      <c r="A51" s="10"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="7"/>
       <c r="F51" s="2"/>
-      <c r="G51" s="4"/>
+      <c r="G51" s="8"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
@@ -1183,13 +1297,13 @@
       <c r="L51" s="2"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="3"/>
+      <c r="A52" s="10"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="7"/>
       <c r="F52" s="2"/>
-      <c r="G52" s="4"/>
+      <c r="G52" s="8"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
@@ -1197,13 +1311,13 @@
       <c r="L52" s="2"/>
     </row>
     <row r="53">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="3"/>
+      <c r="A53" s="10"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="7"/>
       <c r="F53" s="2"/>
-      <c r="G53" s="4"/>
+      <c r="G53" s="8"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
@@ -1211,13 +1325,13 @@
       <c r="L53" s="2"/>
     </row>
     <row r="54">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="3"/>
+      <c r="A54" s="10"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="7"/>
       <c r="F54" s="2"/>
-      <c r="G54" s="4"/>
+      <c r="G54" s="8"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
@@ -1225,13 +1339,13 @@
       <c r="L54" s="2"/>
     </row>
     <row r="55">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="3"/>
+      <c r="A55" s="10"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="7"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="4"/>
+      <c r="G55" s="8"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
@@ -1239,13 +1353,13 @@
       <c r="L55" s="2"/>
     </row>
     <row r="56">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="3"/>
+      <c r="A56" s="10"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="10"/>
+      <c r="E56" s="7"/>
       <c r="F56" s="2"/>
-      <c r="G56" s="4"/>
+      <c r="G56" s="8"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
@@ -1253,13 +1367,13 @@
       <c r="L56" s="2"/>
     </row>
     <row r="57">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="3"/>
+      <c r="A57" s="10"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="10"/>
+      <c r="E57" s="7"/>
       <c r="F57" s="2"/>
-      <c r="G57" s="4"/>
+      <c r="G57" s="8"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
@@ -1267,13 +1381,13 @@
       <c r="L57" s="2"/>
     </row>
     <row r="58">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="3"/>
+      <c r="A58" s="10"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="10"/>
+      <c r="E58" s="7"/>
       <c r="F58" s="2"/>
-      <c r="G58" s="4"/>
+      <c r="G58" s="8"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
@@ -1281,13 +1395,13 @@
       <c r="L58" s="2"/>
     </row>
     <row r="59">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="3"/>
+      <c r="A59" s="10"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="7"/>
       <c r="F59" s="2"/>
-      <c r="G59" s="4"/>
+      <c r="G59" s="8"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
@@ -1295,13 +1409,13 @@
       <c r="L59" s="2"/>
     </row>
     <row r="60">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="3"/>
+      <c r="A60" s="10"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="7"/>
       <c r="F60" s="2"/>
-      <c r="G60" s="4"/>
+      <c r="G60" s="8"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
@@ -1309,13 +1423,13 @@
       <c r="L60" s="2"/>
     </row>
     <row r="61">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="3"/>
+      <c r="A61" s="10"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="7"/>
       <c r="F61" s="2"/>
-      <c r="G61" s="4"/>
+      <c r="G61" s="8"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
@@ -1323,13 +1437,13 @@
       <c r="L61" s="2"/>
     </row>
     <row r="62">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="3"/>
+      <c r="A62" s="10"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="10"/>
+      <c r="E62" s="7"/>
       <c r="F62" s="2"/>
-      <c r="G62" s="4"/>
+      <c r="G62" s="8"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
@@ -1337,13 +1451,13 @@
       <c r="L62" s="2"/>
     </row>
     <row r="63">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="3"/>
+      <c r="A63" s="10"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
+      <c r="E63" s="7"/>
       <c r="F63" s="2"/>
-      <c r="G63" s="4"/>
+      <c r="G63" s="8"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
@@ -1351,13 +1465,13 @@
       <c r="L63" s="2"/>
     </row>
     <row r="64">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="3"/>
+      <c r="A64" s="10"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="10"/>
+      <c r="E64" s="7"/>
       <c r="F64" s="2"/>
-      <c r="G64" s="4"/>
+      <c r="G64" s="8"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
@@ -1365,13 +1479,13 @@
       <c r="L64" s="2"/>
     </row>
     <row r="65">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="3"/>
+      <c r="A65" s="10"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="7"/>
       <c r="F65" s="2"/>
-      <c r="G65" s="4"/>
+      <c r="G65" s="8"/>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
@@ -1379,13 +1493,13 @@
       <c r="L65" s="2"/>
     </row>
     <row r="66">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="3"/>
+      <c r="A66" s="10"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
+      <c r="E66" s="7"/>
       <c r="F66" s="2"/>
-      <c r="G66" s="4"/>
+      <c r="G66" s="8"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
@@ -1393,13 +1507,13 @@
       <c r="L66" s="2"/>
     </row>
     <row r="67">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="3"/>
+      <c r="A67" s="10"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="7"/>
       <c r="F67" s="2"/>
-      <c r="G67" s="4"/>
+      <c r="G67" s="8"/>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
@@ -1407,13 +1521,13 @@
       <c r="L67" s="2"/>
     </row>
     <row r="68">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="3"/>
+      <c r="A68" s="10"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="10"/>
+      <c r="E68" s="7"/>
       <c r="F68" s="2"/>
-      <c r="G68" s="4"/>
+      <c r="G68" s="8"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
@@ -1421,13 +1535,13 @@
       <c r="L68" s="2"/>
     </row>
     <row r="69">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="3"/>
+      <c r="A69" s="10"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="7"/>
       <c r="F69" s="2"/>
-      <c r="G69" s="4"/>
+      <c r="G69" s="8"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
@@ -1435,13 +1549,13 @@
       <c r="L69" s="2"/>
     </row>
     <row r="70">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="3"/>
+      <c r="A70" s="10"/>
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="10"/>
+      <c r="E70" s="7"/>
       <c r="F70" s="2"/>
-      <c r="G70" s="4"/>
+      <c r="G70" s="8"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
@@ -1449,13 +1563,13 @@
       <c r="L70" s="2"/>
     </row>
     <row r="71">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="3"/>
+      <c r="A71" s="10"/>
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="10"/>
+      <c r="E71" s="7"/>
       <c r="F71" s="2"/>
-      <c r="G71" s="4"/>
+      <c r="G71" s="8"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
@@ -1463,13 +1577,13 @@
       <c r="L71" s="2"/>
     </row>
     <row r="72">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="3"/>
+      <c r="A72" s="10"/>
+      <c r="B72" s="10"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="10"/>
+      <c r="E72" s="7"/>
       <c r="F72" s="2"/>
-      <c r="G72" s="4"/>
+      <c r="G72" s="8"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
@@ -1477,13 +1591,13 @@
       <c r="L72" s="2"/>
     </row>
     <row r="73">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="3"/>
+      <c r="A73" s="10"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="10"/>
+      <c r="E73" s="7"/>
       <c r="F73" s="2"/>
-      <c r="G73" s="4"/>
+      <c r="G73" s="8"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
@@ -1491,13 +1605,13 @@
       <c r="L73" s="2"/>
     </row>
     <row r="74">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="3"/>
+      <c r="A74" s="10"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="10"/>
+      <c r="E74" s="7"/>
       <c r="F74" s="2"/>
-      <c r="G74" s="4"/>
+      <c r="G74" s="8"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
@@ -1505,13 +1619,13 @@
       <c r="L74" s="2"/>
     </row>
     <row r="75">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="3"/>
+      <c r="A75" s="10"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="7"/>
       <c r="F75" s="2"/>
-      <c r="G75" s="4"/>
+      <c r="G75" s="8"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
@@ -1519,13 +1633,13 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="3"/>
+      <c r="A76" s="10"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="10"/>
+      <c r="E76" s="7"/>
       <c r="F76" s="2"/>
-      <c r="G76" s="4"/>
+      <c r="G76" s="8"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
@@ -1533,13 +1647,13 @@
       <c r="L76" s="2"/>
     </row>
     <row r="77">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="3"/>
+      <c r="A77" s="10"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="10"/>
+      <c r="E77" s="7"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="4"/>
+      <c r="G77" s="8"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
@@ -1547,13 +1661,13 @@
       <c r="L77" s="2"/>
     </row>
     <row r="78">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="3"/>
+      <c r="A78" s="10"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="10"/>
+      <c r="E78" s="7"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="4"/>
+      <c r="G78" s="8"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
@@ -1561,13 +1675,13 @@
       <c r="L78" s="2"/>
     </row>
     <row r="79">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="3"/>
+      <c r="A79" s="10"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="10"/>
+      <c r="E79" s="7"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="4"/>
+      <c r="G79" s="8"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
@@ -1575,13 +1689,13 @@
       <c r="L79" s="2"/>
     </row>
     <row r="80">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="3"/>
+      <c r="A80" s="10"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="10"/>
+      <c r="E80" s="7"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="4"/>
+      <c r="G80" s="8"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
@@ -1589,13 +1703,13 @@
       <c r="L80" s="2"/>
     </row>
     <row r="81">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
-      <c r="E81" s="3"/>
+      <c r="A81" s="10"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="10"/>
+      <c r="E81" s="7"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="4"/>
+      <c r="G81" s="8"/>
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
@@ -1603,13 +1717,13 @@
       <c r="L81" s="2"/>
     </row>
     <row r="82">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5"/>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
-      <c r="E82" s="3"/>
+      <c r="A82" s="10"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="10"/>
+      <c r="E82" s="7"/>
       <c r="F82" s="2"/>
-      <c r="G82" s="4"/>
+      <c r="G82" s="8"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
@@ -1617,13 +1731,13 @@
       <c r="L82" s="2"/>
     </row>
     <row r="83">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
-      <c r="E83" s="3"/>
+      <c r="A83" s="10"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="10"/>
+      <c r="E83" s="7"/>
       <c r="F83" s="2"/>
-      <c r="G83" s="4"/>
+      <c r="G83" s="8"/>
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
@@ -1631,13 +1745,13 @@
       <c r="L83" s="2"/>
     </row>
     <row r="84">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
-      <c r="C84" s="5"/>
-      <c r="D84" s="5"/>
-      <c r="E84" s="3"/>
+      <c r="A84" s="10"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="10"/>
+      <c r="E84" s="7"/>
       <c r="F84" s="2"/>
-      <c r="G84" s="4"/>
+      <c r="G84" s="8"/>
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
@@ -1645,13 +1759,13 @@
       <c r="L84" s="2"/>
     </row>
     <row r="85">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
-      <c r="E85" s="3"/>
+      <c r="A85" s="10"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="10"/>
+      <c r="E85" s="7"/>
       <c r="F85" s="2"/>
-      <c r="G85" s="4"/>
+      <c r="G85" s="8"/>
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
@@ -1659,13 +1773,13 @@
       <c r="L85" s="2"/>
     </row>
     <row r="86">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
-      <c r="C86" s="5"/>
-      <c r="D86" s="5"/>
-      <c r="E86" s="3"/>
+      <c r="A86" s="10"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+      <c r="E86" s="7"/>
       <c r="F86" s="2"/>
-      <c r="G86" s="4"/>
+      <c r="G86" s="8"/>
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
@@ -1673,13 +1787,13 @@
       <c r="L86" s="2"/>
     </row>
     <row r="87">
-      <c r="A87" s="5"/>
-      <c r="B87" s="5"/>
-      <c r="C87" s="5"/>
-      <c r="D87" s="5"/>
-      <c r="E87" s="3"/>
+      <c r="A87" s="10"/>
+      <c r="B87" s="10"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="10"/>
+      <c r="E87" s="7"/>
       <c r="F87" s="2"/>
-      <c r="G87" s="4"/>
+      <c r="G87" s="8"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
@@ -1687,13 +1801,13 @@
       <c r="L87" s="2"/>
     </row>
     <row r="88">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="5"/>
-      <c r="E88" s="3"/>
+      <c r="A88" s="10"/>
+      <c r="B88" s="10"/>
+      <c r="C88" s="10"/>
+      <c r="D88" s="10"/>
+      <c r="E88" s="7"/>
       <c r="F88" s="2"/>
-      <c r="G88" s="4"/>
+      <c r="G88" s="8"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
@@ -1701,13 +1815,13 @@
       <c r="L88" s="2"/>
     </row>
     <row r="89">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
-      <c r="C89" s="5"/>
-      <c r="D89" s="5"/>
-      <c r="E89" s="3"/>
+      <c r="A89" s="10"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="10"/>
+      <c r="D89" s="10"/>
+      <c r="E89" s="7"/>
       <c r="F89" s="2"/>
-      <c r="G89" s="4"/>
+      <c r="G89" s="8"/>
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
@@ -1715,13 +1829,13 @@
       <c r="L89" s="2"/>
     </row>
     <row r="90">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="5"/>
-      <c r="E90" s="3"/>
+      <c r="A90" s="10"/>
+      <c r="B90" s="10"/>
+      <c r="C90" s="10"/>
+      <c r="D90" s="10"/>
+      <c r="E90" s="7"/>
       <c r="F90" s="2"/>
-      <c r="G90" s="4"/>
+      <c r="G90" s="8"/>
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
@@ -1729,13 +1843,13 @@
       <c r="L90" s="2"/>
     </row>
     <row r="91">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="5"/>
-      <c r="E91" s="3"/>
+      <c r="A91" s="10"/>
+      <c r="B91" s="10"/>
+      <c r="C91" s="10"/>
+      <c r="D91" s="10"/>
+      <c r="E91" s="7"/>
       <c r="F91" s="2"/>
-      <c r="G91" s="4"/>
+      <c r="G91" s="8"/>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
@@ -1743,13 +1857,13 @@
       <c r="L91" s="2"/>
     </row>
     <row r="92">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5"/>
-      <c r="C92" s="5"/>
-      <c r="D92" s="5"/>
-      <c r="E92" s="3"/>
+      <c r="A92" s="10"/>
+      <c r="B92" s="10"/>
+      <c r="C92" s="10"/>
+      <c r="D92" s="10"/>
+      <c r="E92" s="7"/>
       <c r="F92" s="2"/>
-      <c r="G92" s="4"/>
+      <c r="G92" s="8"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
@@ -1757,13 +1871,13 @@
       <c r="L92" s="2"/>
     </row>
     <row r="93">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="5"/>
-      <c r="E93" s="3"/>
+      <c r="A93" s="10"/>
+      <c r="B93" s="10"/>
+      <c r="C93" s="10"/>
+      <c r="D93" s="10"/>
+      <c r="E93" s="7"/>
       <c r="F93" s="2"/>
-      <c r="G93" s="4"/>
+      <c r="G93" s="8"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
@@ -1771,13 +1885,13 @@
       <c r="L93" s="2"/>
     </row>
     <row r="94">
-      <c r="A94" s="5"/>
-      <c r="B94" s="5"/>
-      <c r="C94" s="5"/>
-      <c r="D94" s="5"/>
-      <c r="E94" s="3"/>
+      <c r="A94" s="10"/>
+      <c r="B94" s="10"/>
+      <c r="C94" s="10"/>
+      <c r="D94" s="10"/>
+      <c r="E94" s="7"/>
       <c r="F94" s="2"/>
-      <c r="G94" s="4"/>
+      <c r="G94" s="8"/>
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
@@ -1785,13 +1899,13 @@
       <c r="L94" s="2"/>
     </row>
     <row r="95">
-      <c r="A95" s="5"/>
-      <c r="B95" s="5"/>
-      <c r="C95" s="5"/>
-      <c r="D95" s="5"/>
-      <c r="E95" s="3"/>
+      <c r="A95" s="10"/>
+      <c r="B95" s="10"/>
+      <c r="C95" s="10"/>
+      <c r="D95" s="10"/>
+      <c r="E95" s="7"/>
       <c r="F95" s="2"/>
-      <c r="G95" s="4"/>
+      <c r="G95" s="8"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
@@ -1799,13 +1913,13 @@
       <c r="L95" s="2"/>
     </row>
     <row r="96">
-      <c r="A96" s="5"/>
-      <c r="B96" s="5"/>
-      <c r="C96" s="5"/>
-      <c r="D96" s="5"/>
-      <c r="E96" s="3"/>
+      <c r="A96" s="10"/>
+      <c r="B96" s="10"/>
+      <c r="C96" s="10"/>
+      <c r="D96" s="10"/>
+      <c r="E96" s="7"/>
       <c r="F96" s="2"/>
-      <c r="G96" s="4"/>
+      <c r="G96" s="8"/>
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
@@ -1813,13 +1927,13 @@
       <c r="L96" s="2"/>
     </row>
     <row r="97">
-      <c r="A97" s="5"/>
-      <c r="B97" s="5"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="5"/>
-      <c r="E97" s="3"/>
+      <c r="A97" s="10"/>
+      <c r="B97" s="10"/>
+      <c r="C97" s="10"/>
+      <c r="D97" s="10"/>
+      <c r="E97" s="7"/>
       <c r="F97" s="2"/>
-      <c r="G97" s="4"/>
+      <c r="G97" s="8"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
@@ -1827,13 +1941,13 @@
       <c r="L97" s="2"/>
     </row>
     <row r="98">
-      <c r="A98" s="5"/>
-      <c r="B98" s="5"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="5"/>
-      <c r="E98" s="3"/>
+      <c r="A98" s="10"/>
+      <c r="B98" s="10"/>
+      <c r="C98" s="10"/>
+      <c r="D98" s="10"/>
+      <c r="E98" s="7"/>
       <c r="F98" s="2"/>
-      <c r="G98" s="4"/>
+      <c r="G98" s="8"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
@@ -1841,13 +1955,13 @@
       <c r="L98" s="2"/>
     </row>
     <row r="99">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
-      <c r="C99" s="5"/>
-      <c r="D99" s="5"/>
-      <c r="E99" s="3"/>
+      <c r="A99" s="10"/>
+      <c r="B99" s="10"/>
+      <c r="C99" s="10"/>
+      <c r="D99" s="10"/>
+      <c r="E99" s="7"/>
       <c r="F99" s="2"/>
-      <c r="G99" s="4"/>
+      <c r="G99" s="8"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
@@ -1855,13 +1969,13 @@
       <c r="L99" s="2"/>
     </row>
     <row r="100">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
-      <c r="C100" s="5"/>
-      <c r="D100" s="5"/>
-      <c r="E100" s="3"/>
+      <c r="A100" s="10"/>
+      <c r="B100" s="10"/>
+      <c r="C100" s="10"/>
+      <c r="D100" s="10"/>
+      <c r="E100" s="7"/>
       <c r="F100" s="2"/>
-      <c r="G100" s="4"/>
+      <c r="G100" s="8"/>
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
       <c r="J100" s="2"/>
@@ -1869,13 +1983,13 @@
       <c r="L100" s="2"/>
     </row>
     <row r="101">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
-      <c r="C101" s="5"/>
-      <c r="D101" s="5"/>
-      <c r="E101" s="3"/>
+      <c r="A101" s="10"/>
+      <c r="B101" s="10"/>
+      <c r="C101" s="10"/>
+      <c r="D101" s="10"/>
+      <c r="E101" s="7"/>
       <c r="F101" s="2"/>
-      <c r="G101" s="4"/>
+      <c r="G101" s="8"/>
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
       <c r="J101" s="2"/>
@@ -1908,823 +2022,851 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="7" t="str">
+      <c r="A1" s="14" t="str">
         <v>Package key</v>
       </c>
-      <c r="B1" s="7" t="str">
+      <c r="B1" s="14" t="str">
         <v>Component name</v>
       </c>
-      <c r="C1" s="7" t="str">
+      <c r="C1" s="14" t="str">
         <v>Amount</v>
       </c>
-      <c r="D1" s="7" t="str">
+      <c r="D1" s="14" t="str">
         <v>Frequency</v>
       </c>
-      <c r="E1" s="7" t="str">
+      <c r="E1" s="14" t="str">
         <v>Payable date</v>
       </c>
-      <c r="F1" s="7" t="str">
+      <c r="F1" s="14" t="str">
         <v>Legacy field</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="4" t="str">
+        <v>EXAMPLE-EMP-001</v>
+      </c>
+      <c r="B2" s="4" t="str">
+        <v>Transportation allowance</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D2" s="4" t="str">
+        <v>recurring</v>
+      </c>
+      <c r="E2" s="5" t="str"/>
+      <c r="F2" s="4" t="str">
+        <v>deminimis</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="2"/>
+      <c r="A3" s="4" t="str">
+        <v>EXAMPLE-DUAL-EMP</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>Meal allowance</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D3" s="4" t="str">
+        <v>recurring</v>
+      </c>
+      <c r="E3" s="5" t="str"/>
+      <c r="F3" s="4" t="str"/>
     </row>
     <row r="4">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="2"/>
+      <c r="A4" s="4" t="str">
+        <v>EXAMPLE-DUAL-CONS</v>
+      </c>
+      <c r="B4" s="4" t="str">
+        <v>Project completion fee</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D4" s="4" t="str">
+        <v>one_time</v>
+      </c>
+      <c r="E4" s="5" t="str">
+        <v>2026-12-15</v>
+      </c>
+      <c r="F4" s="4" t="str"/>
     </row>
     <row r="5">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="4"/>
+      <c r="C5" s="8"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="3"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="4"/>
+      <c r="C6" s="8"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="3"/>
+      <c r="E6" s="7"/>
       <c r="F6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
-      <c r="C7" s="4"/>
+      <c r="C7" s="8"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="3"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
-      <c r="C8" s="4"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="3"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="4"/>
+      <c r="C9" s="8"/>
       <c r="D9" s="2"/>
-      <c r="E9" s="3"/>
+      <c r="E9" s="7"/>
       <c r="F9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="4"/>
+      <c r="C10" s="8"/>
       <c r="D10" s="2"/>
-      <c r="E10" s="3"/>
+      <c r="E10" s="7"/>
       <c r="F10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="4"/>
+      <c r="C11" s="8"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="3"/>
+      <c r="E11" s="7"/>
       <c r="F11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
-      <c r="C12" s="4"/>
+      <c r="C12" s="8"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="3"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="4"/>
+      <c r="C13" s="8"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="3"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="8"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="3"/>
+      <c r="E14" s="7"/>
       <c r="F14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="4"/>
+      <c r="C15" s="8"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="3"/>
+      <c r="E15" s="7"/>
       <c r="F15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="4"/>
+      <c r="C16" s="8"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="3"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="4"/>
+      <c r="C17" s="8"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="3"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="4"/>
+      <c r="C18" s="8"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="3"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="4"/>
+      <c r="C19" s="8"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="3"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="4"/>
+      <c r="C20" s="8"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="3"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="4"/>
+      <c r="C21" s="8"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="3"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="4"/>
+      <c r="C22" s="8"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="3"/>
+      <c r="E22" s="7"/>
       <c r="F22" s="2"/>
     </row>
     <row r="23">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="4"/>
+      <c r="C23" s="8"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="3"/>
+      <c r="E23" s="7"/>
       <c r="F23" s="2"/>
     </row>
     <row r="24">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="4"/>
+      <c r="C24" s="8"/>
       <c r="D24" s="2"/>
-      <c r="E24" s="3"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="2"/>
     </row>
     <row r="25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="4"/>
+      <c r="C25" s="8"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="3"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="2"/>
     </row>
     <row r="26">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="4"/>
+      <c r="C26" s="8"/>
       <c r="D26" s="2"/>
-      <c r="E26" s="3"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="2"/>
     </row>
     <row r="27">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="4"/>
+      <c r="C27" s="8"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="3"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="2"/>
     </row>
     <row r="28">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="4"/>
+      <c r="C28" s="8"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="3"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="2"/>
     </row>
     <row r="29">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="4"/>
+      <c r="C29" s="8"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="3"/>
+      <c r="E29" s="7"/>
       <c r="F29" s="2"/>
     </row>
     <row r="30">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="4"/>
+      <c r="C30" s="8"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="3"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="2"/>
     </row>
     <row r="31">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="4"/>
+      <c r="C31" s="8"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="3"/>
+      <c r="E31" s="7"/>
       <c r="F31" s="2"/>
     </row>
     <row r="32">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="4"/>
+      <c r="C32" s="8"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="3"/>
+      <c r="E32" s="7"/>
       <c r="F32" s="2"/>
     </row>
     <row r="33">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="4"/>
+      <c r="C33" s="8"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="3"/>
+      <c r="E33" s="7"/>
       <c r="F33" s="2"/>
     </row>
     <row r="34">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="4"/>
+      <c r="C34" s="8"/>
       <c r="D34" s="2"/>
-      <c r="E34" s="3"/>
+      <c r="E34" s="7"/>
       <c r="F34" s="2"/>
     </row>
     <row r="35">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="4"/>
+      <c r="C35" s="8"/>
       <c r="D35" s="2"/>
-      <c r="E35" s="3"/>
+      <c r="E35" s="7"/>
       <c r="F35" s="2"/>
     </row>
     <row r="36">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="4"/>
+      <c r="C36" s="8"/>
       <c r="D36" s="2"/>
-      <c r="E36" s="3"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="2"/>
     </row>
     <row r="37">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="4"/>
+      <c r="C37" s="8"/>
       <c r="D37" s="2"/>
-      <c r="E37" s="3"/>
+      <c r="E37" s="7"/>
       <c r="F37" s="2"/>
     </row>
     <row r="38">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="4"/>
+      <c r="C38" s="8"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="3"/>
+      <c r="E38" s="7"/>
       <c r="F38" s="2"/>
     </row>
     <row r="39">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="4"/>
+      <c r="C39" s="8"/>
       <c r="D39" s="2"/>
-      <c r="E39" s="3"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="2"/>
     </row>
     <row r="40">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="4"/>
+      <c r="C40" s="8"/>
       <c r="D40" s="2"/>
-      <c r="E40" s="3"/>
+      <c r="E40" s="7"/>
       <c r="F40" s="2"/>
     </row>
     <row r="41">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="4"/>
+      <c r="C41" s="8"/>
       <c r="D41" s="2"/>
-      <c r="E41" s="3"/>
+      <c r="E41" s="7"/>
       <c r="F41" s="2"/>
     </row>
     <row r="42">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="4"/>
+      <c r="C42" s="8"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="3"/>
+      <c r="E42" s="7"/>
       <c r="F42" s="2"/>
     </row>
     <row r="43">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="4"/>
+      <c r="C43" s="8"/>
       <c r="D43" s="2"/>
-      <c r="E43" s="3"/>
+      <c r="E43" s="7"/>
       <c r="F43" s="2"/>
     </row>
     <row r="44">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="4"/>
+      <c r="C44" s="8"/>
       <c r="D44" s="2"/>
-      <c r="E44" s="3"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="2"/>
     </row>
     <row r="45">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="4"/>
+      <c r="C45" s="8"/>
       <c r="D45" s="2"/>
-      <c r="E45" s="3"/>
+      <c r="E45" s="7"/>
       <c r="F45" s="2"/>
     </row>
     <row r="46">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="4"/>
+      <c r="C46" s="8"/>
       <c r="D46" s="2"/>
-      <c r="E46" s="3"/>
+      <c r="E46" s="7"/>
       <c r="F46" s="2"/>
     </row>
     <row r="47">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="4"/>
+      <c r="C47" s="8"/>
       <c r="D47" s="2"/>
-      <c r="E47" s="3"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="2"/>
     </row>
     <row r="48">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
-      <c r="C48" s="4"/>
+      <c r="C48" s="8"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="3"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="2"/>
     </row>
     <row r="49">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
-      <c r="C49" s="4"/>
+      <c r="C49" s="8"/>
       <c r="D49" s="2"/>
-      <c r="E49" s="3"/>
+      <c r="E49" s="7"/>
       <c r="F49" s="2"/>
     </row>
     <row r="50">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
-      <c r="C50" s="4"/>
+      <c r="C50" s="8"/>
       <c r="D50" s="2"/>
-      <c r="E50" s="3"/>
+      <c r="E50" s="7"/>
       <c r="F50" s="2"/>
     </row>
     <row r="51">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
-      <c r="C51" s="4"/>
+      <c r="C51" s="8"/>
       <c r="D51" s="2"/>
-      <c r="E51" s="3"/>
+      <c r="E51" s="7"/>
       <c r="F51" s="2"/>
     </row>
     <row r="52">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
-      <c r="C52" s="4"/>
+      <c r="C52" s="8"/>
       <c r="D52" s="2"/>
-      <c r="E52" s="3"/>
+      <c r="E52" s="7"/>
       <c r="F52" s="2"/>
     </row>
     <row r="53">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
-      <c r="C53" s="4"/>
+      <c r="C53" s="8"/>
       <c r="D53" s="2"/>
-      <c r="E53" s="3"/>
+      <c r="E53" s="7"/>
       <c r="F53" s="2"/>
     </row>
     <row r="54">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
-      <c r="C54" s="4"/>
+      <c r="C54" s="8"/>
       <c r="D54" s="2"/>
-      <c r="E54" s="3"/>
+      <c r="E54" s="7"/>
       <c r="F54" s="2"/>
     </row>
     <row r="55">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
-      <c r="C55" s="4"/>
+      <c r="C55" s="8"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="3"/>
+      <c r="E55" s="7"/>
       <c r="F55" s="2"/>
     </row>
     <row r="56">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
-      <c r="C56" s="4"/>
+      <c r="C56" s="8"/>
       <c r="D56" s="2"/>
-      <c r="E56" s="3"/>
+      <c r="E56" s="7"/>
       <c r="F56" s="2"/>
     </row>
     <row r="57">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
-      <c r="C57" s="4"/>
+      <c r="C57" s="8"/>
       <c r="D57" s="2"/>
-      <c r="E57" s="3"/>
+      <c r="E57" s="7"/>
       <c r="F57" s="2"/>
     </row>
     <row r="58">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
-      <c r="C58" s="4"/>
+      <c r="C58" s="8"/>
       <c r="D58" s="2"/>
-      <c r="E58" s="3"/>
+      <c r="E58" s="7"/>
       <c r="F58" s="2"/>
     </row>
     <row r="59">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
-      <c r="C59" s="4"/>
+      <c r="C59" s="8"/>
       <c r="D59" s="2"/>
-      <c r="E59" s="3"/>
+      <c r="E59" s="7"/>
       <c r="F59" s="2"/>
     </row>
     <row r="60">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
-      <c r="C60" s="4"/>
+      <c r="C60" s="8"/>
       <c r="D60" s="2"/>
-      <c r="E60" s="3"/>
+      <c r="E60" s="7"/>
       <c r="F60" s="2"/>
     </row>
     <row r="61">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
-      <c r="C61" s="4"/>
+      <c r="C61" s="8"/>
       <c r="D61" s="2"/>
-      <c r="E61" s="3"/>
+      <c r="E61" s="7"/>
       <c r="F61" s="2"/>
     </row>
     <row r="62">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
-      <c r="C62" s="4"/>
+      <c r="C62" s="8"/>
       <c r="D62" s="2"/>
-      <c r="E62" s="3"/>
+      <c r="E62" s="7"/>
       <c r="F62" s="2"/>
     </row>
     <row r="63">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
-      <c r="C63" s="4"/>
+      <c r="C63" s="8"/>
       <c r="D63" s="2"/>
-      <c r="E63" s="3"/>
+      <c r="E63" s="7"/>
       <c r="F63" s="2"/>
     </row>
     <row r="64">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
-      <c r="C64" s="4"/>
+      <c r="C64" s="8"/>
       <c r="D64" s="2"/>
-      <c r="E64" s="3"/>
+      <c r="E64" s="7"/>
       <c r="F64" s="2"/>
     </row>
     <row r="65">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
-      <c r="C65" s="4"/>
+      <c r="C65" s="8"/>
       <c r="D65" s="2"/>
-      <c r="E65" s="3"/>
+      <c r="E65" s="7"/>
       <c r="F65" s="2"/>
     </row>
     <row r="66">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
-      <c r="C66" s="4"/>
+      <c r="C66" s="8"/>
       <c r="D66" s="2"/>
-      <c r="E66" s="3"/>
+      <c r="E66" s="7"/>
       <c r="F66" s="2"/>
     </row>
     <row r="67">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
-      <c r="C67" s="4"/>
+      <c r="C67" s="8"/>
       <c r="D67" s="2"/>
-      <c r="E67" s="3"/>
+      <c r="E67" s="7"/>
       <c r="F67" s="2"/>
     </row>
     <row r="68">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
-      <c r="C68" s="4"/>
+      <c r="C68" s="8"/>
       <c r="D68" s="2"/>
-      <c r="E68" s="3"/>
+      <c r="E68" s="7"/>
       <c r="F68" s="2"/>
     </row>
     <row r="69">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
-      <c r="C69" s="4"/>
+      <c r="C69" s="8"/>
       <c r="D69" s="2"/>
-      <c r="E69" s="3"/>
+      <c r="E69" s="7"/>
       <c r="F69" s="2"/>
     </row>
     <row r="70">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
-      <c r="C70" s="4"/>
+      <c r="C70" s="8"/>
       <c r="D70" s="2"/>
-      <c r="E70" s="3"/>
+      <c r="E70" s="7"/>
       <c r="F70" s="2"/>
     </row>
     <row r="71">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
-      <c r="C71" s="4"/>
+      <c r="C71" s="8"/>
       <c r="D71" s="2"/>
-      <c r="E71" s="3"/>
+      <c r="E71" s="7"/>
       <c r="F71" s="2"/>
     </row>
     <row r="72">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
-      <c r="C72" s="4"/>
+      <c r="C72" s="8"/>
       <c r="D72" s="2"/>
-      <c r="E72" s="3"/>
+      <c r="E72" s="7"/>
       <c r="F72" s="2"/>
     </row>
     <row r="73">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
-      <c r="C73" s="4"/>
+      <c r="C73" s="8"/>
       <c r="D73" s="2"/>
-      <c r="E73" s="3"/>
+      <c r="E73" s="7"/>
       <c r="F73" s="2"/>
     </row>
     <row r="74">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
-      <c r="C74" s="4"/>
+      <c r="C74" s="8"/>
       <c r="D74" s="2"/>
-      <c r="E74" s="3"/>
+      <c r="E74" s="7"/>
       <c r="F74" s="2"/>
     </row>
     <row r="75">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
-      <c r="C75" s="4"/>
+      <c r="C75" s="8"/>
       <c r="D75" s="2"/>
-      <c r="E75" s="3"/>
+      <c r="E75" s="7"/>
       <c r="F75" s="2"/>
     </row>
     <row r="76">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
-      <c r="C76" s="4"/>
+      <c r="C76" s="8"/>
       <c r="D76" s="2"/>
-      <c r="E76" s="3"/>
+      <c r="E76" s="7"/>
       <c r="F76" s="2"/>
     </row>
     <row r="77">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
-      <c r="C77" s="4"/>
+      <c r="C77" s="8"/>
       <c r="D77" s="2"/>
-      <c r="E77" s="3"/>
+      <c r="E77" s="7"/>
       <c r="F77" s="2"/>
     </row>
     <row r="78">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
-      <c r="C78" s="4"/>
+      <c r="C78" s="8"/>
       <c r="D78" s="2"/>
-      <c r="E78" s="3"/>
+      <c r="E78" s="7"/>
       <c r="F78" s="2"/>
     </row>
     <row r="79">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
-      <c r="C79" s="4"/>
+      <c r="C79" s="8"/>
       <c r="D79" s="2"/>
-      <c r="E79" s="3"/>
+      <c r="E79" s="7"/>
       <c r="F79" s="2"/>
     </row>
     <row r="80">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
-      <c r="C80" s="4"/>
+      <c r="C80" s="8"/>
       <c r="D80" s="2"/>
-      <c r="E80" s="3"/>
+      <c r="E80" s="7"/>
       <c r="F80" s="2"/>
     </row>
     <row r="81">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
-      <c r="C81" s="4"/>
+      <c r="C81" s="8"/>
       <c r="D81" s="2"/>
-      <c r="E81" s="3"/>
+      <c r="E81" s="7"/>
       <c r="F81" s="2"/>
     </row>
     <row r="82">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
-      <c r="C82" s="4"/>
+      <c r="C82" s="8"/>
       <c r="D82" s="2"/>
-      <c r="E82" s="3"/>
+      <c r="E82" s="7"/>
       <c r="F82" s="2"/>
     </row>
     <row r="83">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
-      <c r="C83" s="4"/>
+      <c r="C83" s="8"/>
       <c r="D83" s="2"/>
-      <c r="E83" s="3"/>
+      <c r="E83" s="7"/>
       <c r="F83" s="2"/>
     </row>
     <row r="84">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
-      <c r="C84" s="4"/>
+      <c r="C84" s="8"/>
       <c r="D84" s="2"/>
-      <c r="E84" s="3"/>
+      <c r="E84" s="7"/>
       <c r="F84" s="2"/>
     </row>
     <row r="85">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
-      <c r="C85" s="4"/>
+      <c r="C85" s="8"/>
       <c r="D85" s="2"/>
-      <c r="E85" s="3"/>
+      <c r="E85" s="7"/>
       <c r="F85" s="2"/>
     </row>
     <row r="86">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
-      <c r="C86" s="4"/>
+      <c r="C86" s="8"/>
       <c r="D86" s="2"/>
-      <c r="E86" s="3"/>
+      <c r="E86" s="7"/>
       <c r="F86" s="2"/>
     </row>
     <row r="87">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
-      <c r="C87" s="4"/>
+      <c r="C87" s="8"/>
       <c r="D87" s="2"/>
-      <c r="E87" s="3"/>
+      <c r="E87" s="7"/>
       <c r="F87" s="2"/>
     </row>
     <row r="88">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
-      <c r="C88" s="4"/>
+      <c r="C88" s="8"/>
       <c r="D88" s="2"/>
-      <c r="E88" s="3"/>
+      <c r="E88" s="7"/>
       <c r="F88" s="2"/>
     </row>
     <row r="89">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
-      <c r="C89" s="4"/>
+      <c r="C89" s="8"/>
       <c r="D89" s="2"/>
-      <c r="E89" s="3"/>
+      <c r="E89" s="7"/>
       <c r="F89" s="2"/>
     </row>
     <row r="90">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
-      <c r="C90" s="4"/>
+      <c r="C90" s="8"/>
       <c r="D90" s="2"/>
-      <c r="E90" s="3"/>
+      <c r="E90" s="7"/>
       <c r="F90" s="2"/>
     </row>
     <row r="91">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
-      <c r="C91" s="4"/>
+      <c r="C91" s="8"/>
       <c r="D91" s="2"/>
-      <c r="E91" s="3"/>
+      <c r="E91" s="7"/>
       <c r="F91" s="2"/>
     </row>
     <row r="92">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
-      <c r="C92" s="4"/>
+      <c r="C92" s="8"/>
       <c r="D92" s="2"/>
-      <c r="E92" s="3"/>
+      <c r="E92" s="7"/>
       <c r="F92" s="2"/>
     </row>
     <row r="93">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
-      <c r="C93" s="4"/>
+      <c r="C93" s="8"/>
       <c r="D93" s="2"/>
-      <c r="E93" s="3"/>
+      <c r="E93" s="7"/>
       <c r="F93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
-      <c r="C94" s="4"/>
+      <c r="C94" s="8"/>
       <c r="D94" s="2"/>
-      <c r="E94" s="3"/>
+      <c r="E94" s="7"/>
       <c r="F94" s="2"/>
     </row>
     <row r="95">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
-      <c r="C95" s="4"/>
+      <c r="C95" s="8"/>
       <c r="D95" s="2"/>
-      <c r="E95" s="3"/>
+      <c r="E95" s="7"/>
       <c r="F95" s="2"/>
     </row>
     <row r="96">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
-      <c r="C96" s="4"/>
+      <c r="C96" s="8"/>
       <c r="D96" s="2"/>
-      <c r="E96" s="3"/>
+      <c r="E96" s="7"/>
       <c r="F96" s="2"/>
     </row>
     <row r="97">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
-      <c r="C97" s="4"/>
+      <c r="C97" s="8"/>
       <c r="D97" s="2"/>
-      <c r="E97" s="3"/>
+      <c r="E97" s="7"/>
       <c r="F97" s="2"/>
     </row>
     <row r="98">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
-      <c r="C98" s="4"/>
+      <c r="C98" s="8"/>
       <c r="D98" s="2"/>
-      <c r="E98" s="3"/>
+      <c r="E98" s="7"/>
       <c r="F98" s="2"/>
     </row>
     <row r="99">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
-      <c r="C99" s="4"/>
+      <c r="C99" s="8"/>
       <c r="D99" s="2"/>
-      <c r="E99" s="3"/>
+      <c r="E99" s="7"/>
       <c r="F99" s="2"/>
     </row>
     <row r="100">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
-      <c r="C100" s="4"/>
+      <c r="C100" s="8"/>
       <c r="D100" s="2"/>
-      <c r="E100" s="3"/>
+      <c r="E100" s="7"/>
       <c r="F100" s="2"/>
     </row>
     <row r="101">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
-      <c r="C101" s="4"/>
+      <c r="C101" s="8"/>
       <c r="D101" s="2"/>
-      <c r="E101" s="3"/>
+      <c r="E101" s="7"/>
       <c r="F101" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clarify pay package inputs and internal keys
</commit_message>
<xml_diff>
--- a/public/templates/Pay-Packages-Batch-Template.xlsx
+++ b/public/templates/Pay-Packages-Batch-Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R51a28096f1b24144"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="R5699423ccae94e05"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R3e16e1c8c64048cf"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R00e0dfdbf82d4a28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="Re3f70a37c62840ac"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R09ba41a36363494c"/>
   </sheets>
 </workbook>
 </file>
@@ -305,153 +305,169 @@
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="1" t="str">
-        <v>1. Fill Packages</v>
+        <v>What is a package?</v>
       </c>
       <c r="B2" s="1" t="str">
-        <v>One row per package. Use a unique Package key, e.g. PKG-001. Maximum 100 packages.</v>
+        <v>One Packages row is one employee’s dated pay arrangement. It is not a company-wide package and you should not invent the salary or fee.</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="1" t="str">
-        <v>2. Identify employee</v>
+        <v>Where do amounts come from?</v>
       </c>
       <c r="B3" s="1" t="str">
-        <v>Copy the exact employee code from Pay Packages. Names are not accepted as identifiers.</v>
+        <v>Copy employee pay from Current HRIS or an approved PAN. Copy professional fees from the approved consultant agreement.</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="1" t="str">
-        <v>3. Choose scope</v>
+        <v>Package key (internal label)</v>
       </c>
       <c r="B4" s="1" t="str">
-        <v>Use the exact business-unit / payroll-group name shown in HRIS.</v>
+        <v>Use one unique label to link a Packages row to its Components, for example PKG-TNG-013-2026-09-01-EMP. It is not a salary-plan name. Never reuse a key across rows.</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="1" t="str">
-        <v>4. Choose stream</v>
+        <v>1. Fill Packages</v>
       </c>
       <c r="B5" s="1" t="str">
-        <v>employee_payroll or professional_fee. Split arrangements use two package rows with different keys.</v>
+        <v>Use one row per employee / pay stream / effective date. Maximum 100 packages.</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="1" t="str">
-        <v>5. Enter date and amount</v>
+        <v>2. Identify employee</v>
       </c>
       <c r="B6" s="1" t="str">
-        <v>Use real dates (YYYY-MM-DD), Monthly / Daily / Hourly, and numeric PHP amounts. Do not use formulas.</v>
+        <v>Copy the exact employee code from Pay Packages. Names are not accepted as identifiers.</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="1" t="str">
-        <v>6. Match salary source</v>
+        <v>3. Choose scope</v>
       </c>
       <c r="B7" s="1" t="str">
-        <v>For employee payroll, base pay, amount unit and legacy allowances must match current HRIS or an approved PAN.</v>
+        <v>Use the exact business-unit / payroll-group name shown in HRIS.</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="1" t="str">
-        <v>7. Approved PAN</v>
+        <v>4. Choose stream</v>
       </c>
       <c r="B8" s="1" t="str">
-        <v>Leave PAN ID blank for current HRIS. Otherwise use the approved PAN UUID and its effective date.</v>
+        <v>employee_payroll or professional_fee. A dual arrangement uses two rows with the same employee code, different keys and different streams.</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="1" t="str">
-        <v>8. References</v>
+        <v>5. Enter date and amount</v>
       </c>
       <c r="B9" s="1" t="str">
-        <v>Source reference and Reason are required, at least 3 characters. Use a supporting document reference.</v>
+        <v>Use real dates (YYYY-MM-DD), Monthly / Daily / Hourly, and numeric PHP amounts. Do not use formulas.</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="1" t="str">
-        <v>9. Professional fees</v>
+        <v>6. Match salary source</v>
       </c>
       <c r="B10" s="1" t="str">
-        <v>Provide a distinct Engagement reference (not employee) and Tax profile reference.</v>
+        <v>For employee payroll, base pay, amount unit and legacy allowances must match current HRIS or an approved PAN.</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="1" t="str">
-        <v>10. Add Components</v>
+        <v>7. Approved PAN</v>
       </c>
       <c r="B11" s="1" t="str">
-        <v>Use the same Package key to attach multiple allowances. Maximum 30 components per package.</v>
+        <v>Leave PAN ID blank for current HRIS. Otherwise use the approved PAN UUID and its effective date.</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="1" t="str">
-        <v>11. Legacy allowances</v>
+        <v>8. References</v>
       </c>
       <c r="B12" s="1" t="str">
-        <v>Use deminimis or reimbursable in Legacy field for existing HRIS allowances; their amounts must match the salary source.</v>
+        <v>Source reference and Reason are required, at least 3 characters. Use a supporting document reference.</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="1" t="str">
-        <v>12. Other components</v>
+        <v>9. Professional fees</v>
       </c>
       <c r="B13" s="1" t="str">
-        <v>Leave Legacy field blank. Frequency is recurring or one_time; one_time requires a Payable date.</v>
+        <v>Provide a distinct Engagement reference (not employee) and Tax profile reference from the approved agreement.</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="1" t="str">
-        <v>13. Upload</v>
+        <v>10. Add Components</v>
       </c>
       <c r="B14" s="1" t="str">
-        <v>Pay Packages → Batch upload pay packages → Upload completed template. Review all row errors, then Save drafts.</v>
+        <v>Use the same Package key to attach multiple allowances. Maximum 30 components per package.</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="1" t="str">
-        <v>14. Examples</v>
+        <v>11. Legacy allowances</v>
       </c>
       <c r="B15" s="1" t="str">
-        <v>Rows whose Package key begins with EXAMPLE- are included for guidance and ignored automatically during upload. Delete them if you prefer a blank sheet.</v>
+        <v>Use deminimis or reimbursable in Legacy field for existing HRIS allowances; their amounts must match the salary source.</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="1" t="str">
-        <v>15. Dual arrangements</v>
+        <v>12. Other components</v>
       </c>
       <c r="B16" s="1" t="str">
-        <v>Use the same Employee code on two rows: one employee_payroll row and one professional_fee row with a distinct Engagement reference.</v>
+        <v>Leave Legacy field blank. Frequency is recurring or one_time; one_time requires a Payable date.</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="1" t="str">
-        <v>16. Review</v>
+        <v>13. Upload</v>
       </c>
       <c r="B17" s="1" t="str">
-        <v>Tax, contribution, proration and 13th-month treatments remain unreviewed. HR must review and authorize drafts.</v>
+        <v>Pay Packages → Batch upload pay packages → Upload completed template. Review all row errors, then Save drafts.</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="1" t="str">
-        <v>17. Existing dates</v>
+        <v>14. Examples</v>
       </c>
       <c r="B18" s="1" t="str">
-        <v>Imports reject existing non-rejected packages for the same employee, engagement and effective date. Use the individual form for corrections.</v>
+        <v>Rows whose Package key begins with EXAMPLE- are included for guidance and ignored automatically during upload. Replace them with real employee rows before saving.</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="1" t="str">
-        <v>18. Interrupted save</v>
+        <v>15. Review</v>
       </c>
       <c r="B19" s="1" t="str">
-        <v>Saving stops at the first failure. Earlier drafts remain saved. Check existing drafts before uploading only remaining rows.</v>
+        <v>Tax, contribution, proration and 13th-month treatments remain unreviewed. HR must review and authorize drafts.</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="1" t="str">
+        <v>16. Existing dates</v>
+      </c>
+      <c r="B20" s="1" t="str">
+        <v>Imports reject existing non-rejected packages for the same employee, engagement and effective date. Use the individual form for corrections.</v>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="1" t="str">
+        <v>17. Interrupted save</v>
+      </c>
+      <c r="B21" s="1" t="str">
+        <v>Saving stops at the first failure. Earlier drafts remain saved. Check existing drafts before uploading only remaining rows.</v>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="1" t="str">
         <v>Available BU names</v>
       </c>
-      <c r="B20" s="1" t="str">
+      <c r="B22" s="1" t="str">
         <v>The Fun Roof; The Dessert Museum; Gootopia SM North Edsa; Bakebe - S Maison; Bakebe - SM Aura; Gootopia - SM MOA; Inflatable Island Beach Club; TNG (Corporation)</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Prevent real employee rows from being treated as examples
</commit_message>
<xml_diff>
--- a/public/templates/Pay-Packages-Batch-Template.xlsx
+++ b/public/templates/Pay-Packages-Batch-Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R00e0dfdbf82d4a28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="Re3f70a37c62840ac"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R09ba41a36363494c"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rc3f93046008c42ee"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="R0fdb40a204794635"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R28a4937bef414bcc"/>
   </sheets>
 </workbook>
 </file>
@@ -436,7 +436,7 @@
         <v>14. Examples</v>
       </c>
       <c r="B18" s="1" t="str">
-        <v>Rows whose Package key begins with EXAMPLE- are included for guidance and ignored automatically during upload. Replace them with real employee rows before saving.</v>
+        <v>The template’s dummy rows use TNG-EXAMPLE-... employee codes and are ignored automatically. Replace them with real employee rows before saving; do not reuse their sample keys for real employees.</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Process real rows that reuse example package keys
Skip only clearly marked dummy rows; process real employee rows even if an example package key is reused.
</commit_message>
<xml_diff>
--- a/public/templates/Pay-Packages-Batch-Template.xlsx
+++ b/public/templates/Pay-Packages-Batch-Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R00e0dfdbf82d4a28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="Re3f70a37c62840ac"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R09ba41a36363494c"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rc3f93046008c42ee"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="2" r:id="R0fdb40a204794635"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components" sheetId="3" r:id="R28a4937bef414bcc"/>
   </sheets>
 </workbook>
 </file>
@@ -436,7 +436,7 @@
         <v>14. Examples</v>
       </c>
       <c r="B18" s="1" t="str">
-        <v>Rows whose Package key begins with EXAMPLE- are included for guidance and ignored automatically during upload. Replace them with real employee rows before saving.</v>
+        <v>The template’s dummy rows use TNG-EXAMPLE-... employee codes and are ignored automatically. Replace them with real employee rows before saving; do not reuse their sample keys for real employees.</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Fix scoped HR Manager package editing and explain template fields
</commit_message>
<xml_diff>
--- a/public/templates/Pay-Packages-Batch-Template.xlsx
+++ b/public/templates/Pay-Packages-Batch-Template.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pay Input" sheetId="1" r:id="Rc3efa320affb414b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="2" r:id="R795dde1e9e0b4341"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" r:id="R857c4a2177e34c04"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pay Input" sheetId="1" r:id="R9f1bc037d3784d46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="2" r:id="R7df0632424eb4be9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" r:id="R45eadc73e1c34a9b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="Rd583902c51b84bee"/>
   </sheets>
 </workbook>
 </file>
@@ -3767,10 +3768,10 @@
       <formula1>"Monthly,Daily,Hourly"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I101">
-      <formula1>"Gross salary,Net - company covers tax,Net - company covers tax and employee shares,Custom - needs review"</formula1>
+      <formula1>"Gross salary,Company pays income tax,Company pays income tax and employee contributions,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="L2:L101">
-      <formula1>"Standard - Finance reviews,Exemption requested - evidence required,Custom - needs review"</formula1>
+      <formula1>"Normal tax calculation,Exemption requested - evidence required,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="Z2:Z101">
       <formula1>"Current HRIS record,Approved PAN,Approved consultant agreement"</formula1>
@@ -3964,7 +3965,7 @@
       <c r="J2" s="19"/>
       <c r="K2" s="17" t="str"/>
       <c r="L2" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M2" s="17" t="str"/>
       <c r="N2" s="17" t="str">
@@ -4024,7 +4025,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="17" t="str">
-        <v>Net - company covers tax</v>
+        <v>Company pays income tax</v>
       </c>
       <c r="J3" s="19" t="n">
         <v>30000</v>
@@ -4033,7 +4034,7 @@
         <v>Approved agreement / sample only</v>
       </c>
       <c r="L3" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M3" s="17" t="str"/>
       <c r="N3" s="17" t="str"/>
@@ -4087,7 +4088,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="17" t="str">
-        <v>Net - company covers tax and employee shares</v>
+        <v>Company pays income tax and employee contributions</v>
       </c>
       <c r="J4" s="19" t="n">
         <v>30000</v>
@@ -4096,7 +4097,7 @@
         <v>Approved agreement / sample only</v>
       </c>
       <c r="L4" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M4" s="17" t="str"/>
       <c r="N4" s="17" t="str"/>
@@ -4155,7 +4156,7 @@
       <c r="J5" s="19"/>
       <c r="K5" s="17" t="str"/>
       <c r="L5" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M5" s="17" t="str"/>
       <c r="N5" s="17" t="str"/>
@@ -4214,7 +4215,7 @@
       <c r="J6" s="19"/>
       <c r="K6" s="17" t="str"/>
       <c r="L6" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M6" s="17" t="str"/>
       <c r="N6" s="17" t="str">
@@ -4266,10 +4267,10 @@
       <formula1>"Monthly,Daily,Hourly"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I6">
-      <formula1>"Gross salary,Net - company covers tax,Net - company covers tax and employee shares,Custom - needs review"</formula1>
+      <formula1>"Gross salary,Company pays income tax,Company pays income tax and employee contributions,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="L2:L6">
-      <formula1>"Standard - Finance reviews,Exemption requested - evidence required,Custom - needs review"</formula1>
+      <formula1>"Normal tax calculation,Exemption requested - evidence required,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="Z2:Z6">
       <formula1>"Current HRIS record,Approved PAN,Approved consultant agreement"</formula1>
@@ -4321,7 +4322,7 @@
         <v>START HERE</v>
       </c>
       <c r="B2" s="20" t="str">
-        <v>Fill Pay Input only. Use Examples as a guide; replace sample details with approved facts. Upload on Payroll → Pay Packages, review the preview, then save drafts. Never relabel a net agreement as Gross.</v>
+        <v>Fill Pay Input only. Field Guide explains EVERY field and gives exact choices/examples. Use Examples as a guide; replace sample details with approved facts. Upload on Payroll → Pay Packages, review the preview, then save drafts. Never relabel a net agreement as Gross.</v>
       </c>
     </row>
     <row r="3" ht="56" customHeight="1">
@@ -4474,6 +4475,469 @@
       </c>
       <c r="B21" s="20" t="str">
         <v>https://www.philhealth.gov.ph/partners/employers/pay_procedures.php</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="76" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Field name</v>
+      </c>
+      <c r="B1" s="4" t="str">
+        <v>When to fill</v>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v>What to enter</v>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v>Example / choice</v>
+      </c>
+    </row>
+    <row r="2" ht="76" customHeight="1">
+      <c r="A2" s="20" t="str">
+        <v>Employee code</v>
+      </c>
+      <c r="B2" s="20" t="str">
+        <v>Required</v>
+      </c>
+      <c r="C2" s="20" t="str">
+        <v>Copy from Employee codes you can access on the upload page. Do not invent an ID. Missing employee? Register in HRIS first.</v>
+      </c>
+      <c r="D2" s="20" t="str">
+        <v>TNG-EXAMPLE-001 (example only)</v>
+      </c>
+    </row>
+    <row r="3" ht="76" customHeight="1">
+      <c r="A3" s="20" t="str">
+        <v>Business unit</v>
+      </c>
+      <c r="B3" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C3" s="20" t="str">
+        <v>Choose the employee payroll group exactly as listed.</v>
+      </c>
+      <c r="D3" s="20" t="str">
+        <v>The Fun Roof</v>
+      </c>
+    </row>
+    <row r="4" ht="76" customHeight="1">
+      <c r="A4" s="20" t="str">
+        <v>Pay type</v>
+      </c>
+      <c r="B4" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C4" s="20" t="str">
+        <v>Employee salary; a separate consulting engagement needs another row.</v>
+      </c>
+      <c r="D4" s="20" t="str">
+        <v>Employee salary</v>
+      </c>
+    </row>
+    <row r="5" ht="76" customHeight="1">
+      <c r="A5" s="20" t="str">
+        <v>Effective date</v>
+      </c>
+      <c r="B5" s="20" t="str">
+        <v>Required date</v>
+      </c>
+      <c r="C5" s="20" t="str">
+        <v>Actual approved start date of this pay arrangement, not automatically the hire date.</v>
+      </c>
+      <c r="D5" s="20" t="str">
+        <v>2026-09-01</v>
+      </c>
+    </row>
+    <row r="6" ht="76" customHeight="1">
+      <c r="A6" s="20" t="str">
+        <v>Amount unit</v>
+      </c>
+      <c r="B6" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C6" s="20" t="str">
+        <v>Basis of the approved amount. Daily/hourly is not monthly salary.</v>
+      </c>
+      <c r="D6" s="20" t="str">
+        <v>Monthly</v>
+      </c>
+    </row>
+    <row r="7" ht="76" customHeight="1">
+      <c r="A7" s="20" t="str">
+        <v>Approved basic pay / fee</v>
+      </c>
+      <c r="B7" s="20" t="str">
+        <v>Required amount</v>
+      </c>
+      <c r="C7" s="20" t="str">
+        <v>Copy approved basic pay from HRIS/PAN. Do not replace it with guessed gross-up.</v>
+      </c>
+      <c r="D7" s="20" t="str">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="8" ht="76" customHeight="1">
+      <c r="A8" s="20" t="str">
+        <v>Existing de minimis</v>
+      </c>
+      <c r="B8" s="20" t="str">
+        <v>If recorded in HRIS</v>
+      </c>
+      <c r="C8" s="20" t="str">
+        <v>Must exactly match the existing approved allowance; do not repeat under Extras.</v>
+      </c>
+      <c r="D8" s="20" t="str">
+        <v>1500 (example only)</v>
+      </c>
+    </row>
+    <row r="9" ht="76" customHeight="1">
+      <c r="A9" s="20" t="str">
+        <v>Existing reimbursable</v>
+      </c>
+      <c r="B9" s="20" t="str">
+        <v>If recorded in HRIS</v>
+      </c>
+      <c r="C9" s="20" t="str">
+        <v>Must exactly match HRIS/PAN; blank means none in this upload.</v>
+      </c>
+      <c r="D9" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="10" ht="76" customHeight="1">
+      <c r="A10" s="20" t="str">
+        <v>Salary arrangement</v>
+      </c>
+      <c r="B10" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C10" s="20" t="str">
+        <v>Gross salary = employee deductions apply. Company pays income tax = tax covered only. Company pays income tax and employee contributions = both covered.</v>
+      </c>
+      <c r="D10" s="20" t="str">
+        <v>Choose the approved arrangement</v>
+      </c>
+    </row>
+    <row r="11" ht="76" customHeight="1">
+      <c r="A11" s="20" t="str">
+        <v>Agreed net amount</v>
+      </c>
+      <c r="B11" s="20" t="str">
+        <v>Net arrangements only</v>
+      </c>
+      <c r="C11" s="20" t="str">
+        <v>Approved target for this payment unit. Tax-only target is before employee contributions; tax-plus-contributions target is after both, before loans/other deductions.</v>
+      </c>
+      <c r="D11" s="20" t="str">
+        <v>30000 (example only)</v>
+      </c>
+    </row>
+    <row r="12" ht="76" customHeight="1">
+      <c r="A12" s="20" t="str">
+        <v>Arrangement document</v>
+      </c>
+      <c r="B12" s="20" t="str">
+        <v>Net/custom only</v>
+      </c>
+      <c r="C12" s="20" t="str">
+        <v>Approved JO, PAN or signed agreement explicitly stating net terms. Enter title/reference and date. A generic JO without net terms is insufficient.</v>
+      </c>
+      <c r="D12" s="20" t="str">
+        <v>Approved JO for [employee], [date], section [x] confirming tax coverage</v>
+      </c>
+    </row>
+    <row r="13" ht="76" customHeight="1">
+      <c r="A13" s="20" t="str">
+        <v>Tax treatment</v>
+      </c>
+      <c r="B13" s="20" t="str">
+        <v>Dropdown; blank = normal</v>
+      </c>
+      <c r="C13" s="20" t="str">
+        <v>Choose Normal tax calculation even when company pays tax. Exemption requires a genuine separate basis and evidence.</v>
+      </c>
+      <c r="D13" s="20" t="str">
+        <v>Normal tax calculation</v>
+      </c>
+    </row>
+    <row r="14" ht="76" customHeight="1">
+      <c r="A14" s="20" t="str">
+        <v>Exemption / tax basis</v>
+      </c>
+      <c r="B14" s="20" t="str">
+        <v>Only exemption/custom</v>
+      </c>
+      <c r="C14" s="20" t="str">
+        <v>Actual supporting basis and document; do not use net salary as the basis.</v>
+      </c>
+      <c r="D14" s="20" t="str">
+        <v>Leave blank for normal tax calculation</v>
+      </c>
+    </row>
+    <row r="15" ht="76" customHeight="1">
+      <c r="A15" s="20" t="str">
+        <v>Extra 1 name</v>
+      </c>
+      <c r="B15" s="20" t="str">
+        <v>Optional dropdown or custom</v>
+      </c>
+      <c r="C15" s="20" t="str">
+        <v>Name an additional approved component. Do not repeat existing allowances.</v>
+      </c>
+      <c r="D15" s="20" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="16" ht="76" customHeight="1">
+      <c r="A16" s="20" t="str">
+        <v>Extra 1 amount</v>
+      </c>
+      <c r="B16" s="20" t="str">
+        <v>When Extra name is filled</v>
+      </c>
+      <c r="C16" s="20" t="str">
+        <v>Approved component amount.</v>
+      </c>
+      <c r="D16" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="17" ht="76" customHeight="1">
+      <c r="A17" s="20" t="str">
+        <v>Extra 1 frequency</v>
+      </c>
+      <c r="B17" s="20" t="str">
+        <v>Dropdown</v>
+      </c>
+      <c r="C17" s="20" t="str">
+        <v>Recurring uses the package amount unit. One time requires a payable date.</v>
+      </c>
+      <c r="D17" s="20" t="str">
+        <v>Recurring</v>
+      </c>
+    </row>
+    <row r="18" ht="76" customHeight="1">
+      <c r="A18" s="20" t="str">
+        <v>Extra 1 payable date</v>
+      </c>
+      <c r="B18" s="20" t="str">
+        <v>One time only</v>
+      </c>
+      <c r="C18" s="20" t="str">
+        <v>Approved payment date. Leave blank for recurring.</v>
+      </c>
+      <c r="D18" s="20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="19" ht="76" customHeight="1">
+      <c r="A19" s="20" t="str">
+        <v>Extra 2 name</v>
+      </c>
+      <c r="B19" s="20" t="str">
+        <v>Optional dropdown or custom</v>
+      </c>
+      <c r="C19" s="20" t="str">
+        <v>Name an additional approved component. Do not repeat existing allowances.</v>
+      </c>
+      <c r="D19" s="20" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="20" ht="76" customHeight="1">
+      <c r="A20" s="20" t="str">
+        <v>Extra 2 amount</v>
+      </c>
+      <c r="B20" s="20" t="str">
+        <v>When Extra name is filled</v>
+      </c>
+      <c r="C20" s="20" t="str">
+        <v>Approved component amount.</v>
+      </c>
+      <c r="D20" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="21" ht="76" customHeight="1">
+      <c r="A21" s="20" t="str">
+        <v>Extra 2 frequency</v>
+      </c>
+      <c r="B21" s="20" t="str">
+        <v>Dropdown</v>
+      </c>
+      <c r="C21" s="20" t="str">
+        <v>Recurring uses the package amount unit. One time requires a payable date.</v>
+      </c>
+      <c r="D21" s="20" t="str">
+        <v>Recurring</v>
+      </c>
+    </row>
+    <row r="22" ht="76" customHeight="1">
+      <c r="A22" s="20" t="str">
+        <v>Extra 2 payable date</v>
+      </c>
+      <c r="B22" s="20" t="str">
+        <v>One time only</v>
+      </c>
+      <c r="C22" s="20" t="str">
+        <v>Approved payment date. Leave blank for recurring.</v>
+      </c>
+      <c r="D22" s="20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="23" ht="76" customHeight="1">
+      <c r="A23" s="20" t="str">
+        <v>Extra 3 name</v>
+      </c>
+      <c r="B23" s="20" t="str">
+        <v>Optional dropdown or custom</v>
+      </c>
+      <c r="C23" s="20" t="str">
+        <v>Name an additional approved component. Do not repeat existing allowances.</v>
+      </c>
+      <c r="D23" s="20" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="24" ht="76" customHeight="1">
+      <c r="A24" s="20" t="str">
+        <v>Extra 3 amount</v>
+      </c>
+      <c r="B24" s="20" t="str">
+        <v>When Extra name is filled</v>
+      </c>
+      <c r="C24" s="20" t="str">
+        <v>Approved component amount.</v>
+      </c>
+      <c r="D24" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="25" ht="76" customHeight="1">
+      <c r="A25" s="20" t="str">
+        <v>Extra 3 frequency</v>
+      </c>
+      <c r="B25" s="20" t="str">
+        <v>Dropdown</v>
+      </c>
+      <c r="C25" s="20" t="str">
+        <v>Recurring uses the package amount unit. One time requires a payable date.</v>
+      </c>
+      <c r="D25" s="20" t="str">
+        <v>Recurring</v>
+      </c>
+    </row>
+    <row r="26" ht="76" customHeight="1">
+      <c r="A26" s="20" t="str">
+        <v>Extra 3 payable date</v>
+      </c>
+      <c r="B26" s="20" t="str">
+        <v>One time only</v>
+      </c>
+      <c r="C26" s="20" t="str">
+        <v>Approved payment date. Leave blank for recurring.</v>
+      </c>
+      <c r="D26" s="20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="27" ht="76" customHeight="1">
+      <c r="A27" s="20" t="str">
+        <v>Salary source</v>
+      </c>
+      <c r="B27" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C27" s="20" t="str">
+        <v>Where approved salary comes from.</v>
+      </c>
+      <c r="D27" s="20" t="str">
+        <v>Current HRIS record</v>
+      </c>
+    </row>
+    <row r="28" ht="76" customHeight="1">
+      <c r="A28" s="20" t="str">
+        <v>PAN ID (if applicable)</v>
+      </c>
+      <c r="B28" s="20" t="str">
+        <v>Approved PAN only</v>
+      </c>
+      <c r="C28" s="20" t="str">
+        <v>Copy actual PAN record ID from HRIS; otherwise leave blank.</v>
+      </c>
+      <c r="D28" s="20" t="str">
+        <v>Leave blank for Current HRIS record</v>
+      </c>
+    </row>
+    <row r="29" ht="76" customHeight="1">
+      <c r="A29" s="20" t="str">
+        <v>Source document / note</v>
+      </c>
+      <c r="B29" s="20" t="str">
+        <v>Optional descriptive text</v>
+      </c>
+      <c r="C29" s="20" t="str">
+        <v>Actual source reference. Blank uses Salary source.</v>
+      </c>
+      <c r="D29" s="20" t="str">
+        <v>Current HRIS record checked on [date]</v>
+      </c>
+    </row>
+    <row r="30" ht="76" customHeight="1">
+      <c r="A30" s="20" t="str">
+        <v>Reason for this record</v>
+      </c>
+      <c r="B30" s="20" t="str">
+        <v>Required dropdown or text</v>
+      </c>
+      <c r="C30" s="20" t="str">
+        <v>Why this package is being recorded.</v>
+      </c>
+      <c r="D30" s="20" t="str">
+        <v>Initial setup</v>
+      </c>
+    </row>
+    <row r="31" ht="76" customHeight="1">
+      <c r="A31" s="20" t="str">
+        <v>Consultant agreement</v>
+      </c>
+      <c r="B31" s="20" t="str">
+        <v>Consultant row only</v>
+      </c>
+      <c r="C31" s="20" t="str">
+        <v>Actual distinct consulting engagement reference, not employee salary agreement.</v>
+      </c>
+      <c r="D31" s="20" t="str">
+        <v>Signed consulting agreement [reference/date]</v>
+      </c>
+    </row>
+    <row r="32" ht="76" customHeight="1">
+      <c r="A32" s="20" t="str">
+        <v>Consultant tax document</v>
+      </c>
+      <c r="B32" s="20" t="str">
+        <v>Consultant row only</v>
+      </c>
+      <c r="C32" s="20" t="str">
+        <v>Actual reviewed consultant withholding/tax-profile reference.</v>
+      </c>
+      <c r="D32" s="20" t="str">
+        <v>Finance-reviewed tax profile [reference]</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix scoped HR Manager package editing and explain template fields (#41)
</commit_message>
<xml_diff>
--- a/public/templates/Pay-Packages-Batch-Template.xlsx
+++ b/public/templates/Pay-Packages-Batch-Template.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pay Input" sheetId="1" r:id="Rc3efa320affb414b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="2" r:id="R795dde1e9e0b4341"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" r:id="R857c4a2177e34c04"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pay Input" sheetId="1" r:id="R9f1bc037d3784d46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="2" r:id="R7df0632424eb4be9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" r:id="R45eadc73e1c34a9b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="Rd583902c51b84bee"/>
   </sheets>
 </workbook>
 </file>
@@ -3767,10 +3768,10 @@
       <formula1>"Monthly,Daily,Hourly"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I101">
-      <formula1>"Gross salary,Net - company covers tax,Net - company covers tax and employee shares,Custom - needs review"</formula1>
+      <formula1>"Gross salary,Company pays income tax,Company pays income tax and employee contributions,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="L2:L101">
-      <formula1>"Standard - Finance reviews,Exemption requested - evidence required,Custom - needs review"</formula1>
+      <formula1>"Normal tax calculation,Exemption requested - evidence required,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="Z2:Z101">
       <formula1>"Current HRIS record,Approved PAN,Approved consultant agreement"</formula1>
@@ -3964,7 +3965,7 @@
       <c r="J2" s="19"/>
       <c r="K2" s="17" t="str"/>
       <c r="L2" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M2" s="17" t="str"/>
       <c r="N2" s="17" t="str">
@@ -4024,7 +4025,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="17" t="str">
-        <v>Net - company covers tax</v>
+        <v>Company pays income tax</v>
       </c>
       <c r="J3" s="19" t="n">
         <v>30000</v>
@@ -4033,7 +4034,7 @@
         <v>Approved agreement / sample only</v>
       </c>
       <c r="L3" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M3" s="17" t="str"/>
       <c r="N3" s="17" t="str"/>
@@ -4087,7 +4088,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="17" t="str">
-        <v>Net - company covers tax and employee shares</v>
+        <v>Company pays income tax and employee contributions</v>
       </c>
       <c r="J4" s="19" t="n">
         <v>30000</v>
@@ -4096,7 +4097,7 @@
         <v>Approved agreement / sample only</v>
       </c>
       <c r="L4" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M4" s="17" t="str"/>
       <c r="N4" s="17" t="str"/>
@@ -4155,7 +4156,7 @@
       <c r="J5" s="19"/>
       <c r="K5" s="17" t="str"/>
       <c r="L5" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M5" s="17" t="str"/>
       <c r="N5" s="17" t="str"/>
@@ -4214,7 +4215,7 @@
       <c r="J6" s="19"/>
       <c r="K6" s="17" t="str"/>
       <c r="L6" s="17" t="str">
-        <v>Standard - Finance reviews</v>
+        <v>Normal tax calculation</v>
       </c>
       <c r="M6" s="17" t="str"/>
       <c r="N6" s="17" t="str">
@@ -4266,10 +4267,10 @@
       <formula1>"Monthly,Daily,Hourly"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I6">
-      <formula1>"Gross salary,Net - company covers tax,Net - company covers tax and employee shares,Custom - needs review"</formula1>
+      <formula1>"Gross salary,Company pays income tax,Company pays income tax and employee contributions,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="L2:L6">
-      <formula1>"Standard - Finance reviews,Exemption requested - evidence required,Custom - needs review"</formula1>
+      <formula1>"Normal tax calculation,Exemption requested - evidence required,Custom - needs review"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="Z2:Z6">
       <formula1>"Current HRIS record,Approved PAN,Approved consultant agreement"</formula1>
@@ -4321,7 +4322,7 @@
         <v>START HERE</v>
       </c>
       <c r="B2" s="20" t="str">
-        <v>Fill Pay Input only. Use Examples as a guide; replace sample details with approved facts. Upload on Payroll → Pay Packages, review the preview, then save drafts. Never relabel a net agreement as Gross.</v>
+        <v>Fill Pay Input only. Field Guide explains EVERY field and gives exact choices/examples. Use Examples as a guide; replace sample details with approved facts. Upload on Payroll → Pay Packages, review the preview, then save drafts. Never relabel a net agreement as Gross.</v>
       </c>
     </row>
     <row r="3" ht="56" customHeight="1">
@@ -4474,6 +4475,469 @@
       </c>
       <c r="B21" s="20" t="str">
         <v>https://www.philhealth.gov.ph/partners/employers/pay_procedures.php</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="76" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Field name</v>
+      </c>
+      <c r="B1" s="4" t="str">
+        <v>When to fill</v>
+      </c>
+      <c r="C1" s="4" t="str">
+        <v>What to enter</v>
+      </c>
+      <c r="D1" s="4" t="str">
+        <v>Example / choice</v>
+      </c>
+    </row>
+    <row r="2" ht="76" customHeight="1">
+      <c r="A2" s="20" t="str">
+        <v>Employee code</v>
+      </c>
+      <c r="B2" s="20" t="str">
+        <v>Required</v>
+      </c>
+      <c r="C2" s="20" t="str">
+        <v>Copy from Employee codes you can access on the upload page. Do not invent an ID. Missing employee? Register in HRIS first.</v>
+      </c>
+      <c r="D2" s="20" t="str">
+        <v>TNG-EXAMPLE-001 (example only)</v>
+      </c>
+    </row>
+    <row r="3" ht="76" customHeight="1">
+      <c r="A3" s="20" t="str">
+        <v>Business unit</v>
+      </c>
+      <c r="B3" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C3" s="20" t="str">
+        <v>Choose the employee payroll group exactly as listed.</v>
+      </c>
+      <c r="D3" s="20" t="str">
+        <v>The Fun Roof</v>
+      </c>
+    </row>
+    <row r="4" ht="76" customHeight="1">
+      <c r="A4" s="20" t="str">
+        <v>Pay type</v>
+      </c>
+      <c r="B4" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C4" s="20" t="str">
+        <v>Employee salary; a separate consulting engagement needs another row.</v>
+      </c>
+      <c r="D4" s="20" t="str">
+        <v>Employee salary</v>
+      </c>
+    </row>
+    <row r="5" ht="76" customHeight="1">
+      <c r="A5" s="20" t="str">
+        <v>Effective date</v>
+      </c>
+      <c r="B5" s="20" t="str">
+        <v>Required date</v>
+      </c>
+      <c r="C5" s="20" t="str">
+        <v>Actual approved start date of this pay arrangement, not automatically the hire date.</v>
+      </c>
+      <c r="D5" s="20" t="str">
+        <v>2026-09-01</v>
+      </c>
+    </row>
+    <row r="6" ht="76" customHeight="1">
+      <c r="A6" s="20" t="str">
+        <v>Amount unit</v>
+      </c>
+      <c r="B6" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C6" s="20" t="str">
+        <v>Basis of the approved amount. Daily/hourly is not monthly salary.</v>
+      </c>
+      <c r="D6" s="20" t="str">
+        <v>Monthly</v>
+      </c>
+    </row>
+    <row r="7" ht="76" customHeight="1">
+      <c r="A7" s="20" t="str">
+        <v>Approved basic pay / fee</v>
+      </c>
+      <c r="B7" s="20" t="str">
+        <v>Required amount</v>
+      </c>
+      <c r="C7" s="20" t="str">
+        <v>Copy approved basic pay from HRIS/PAN. Do not replace it with guessed gross-up.</v>
+      </c>
+      <c r="D7" s="20" t="str">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="8" ht="76" customHeight="1">
+      <c r="A8" s="20" t="str">
+        <v>Existing de minimis</v>
+      </c>
+      <c r="B8" s="20" t="str">
+        <v>If recorded in HRIS</v>
+      </c>
+      <c r="C8" s="20" t="str">
+        <v>Must exactly match the existing approved allowance; do not repeat under Extras.</v>
+      </c>
+      <c r="D8" s="20" t="str">
+        <v>1500 (example only)</v>
+      </c>
+    </row>
+    <row r="9" ht="76" customHeight="1">
+      <c r="A9" s="20" t="str">
+        <v>Existing reimbursable</v>
+      </c>
+      <c r="B9" s="20" t="str">
+        <v>If recorded in HRIS</v>
+      </c>
+      <c r="C9" s="20" t="str">
+        <v>Must exactly match HRIS/PAN; blank means none in this upload.</v>
+      </c>
+      <c r="D9" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="10" ht="76" customHeight="1">
+      <c r="A10" s="20" t="str">
+        <v>Salary arrangement</v>
+      </c>
+      <c r="B10" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C10" s="20" t="str">
+        <v>Gross salary = employee deductions apply. Company pays income tax = tax covered only. Company pays income tax and employee contributions = both covered.</v>
+      </c>
+      <c r="D10" s="20" t="str">
+        <v>Choose the approved arrangement</v>
+      </c>
+    </row>
+    <row r="11" ht="76" customHeight="1">
+      <c r="A11" s="20" t="str">
+        <v>Agreed net amount</v>
+      </c>
+      <c r="B11" s="20" t="str">
+        <v>Net arrangements only</v>
+      </c>
+      <c r="C11" s="20" t="str">
+        <v>Approved target for this payment unit. Tax-only target is before employee contributions; tax-plus-contributions target is after both, before loans/other deductions.</v>
+      </c>
+      <c r="D11" s="20" t="str">
+        <v>30000 (example only)</v>
+      </c>
+    </row>
+    <row r="12" ht="76" customHeight="1">
+      <c r="A12" s="20" t="str">
+        <v>Arrangement document</v>
+      </c>
+      <c r="B12" s="20" t="str">
+        <v>Net/custom only</v>
+      </c>
+      <c r="C12" s="20" t="str">
+        <v>Approved JO, PAN or signed agreement explicitly stating net terms. Enter title/reference and date. A generic JO without net terms is insufficient.</v>
+      </c>
+      <c r="D12" s="20" t="str">
+        <v>Approved JO for [employee], [date], section [x] confirming tax coverage</v>
+      </c>
+    </row>
+    <row r="13" ht="76" customHeight="1">
+      <c r="A13" s="20" t="str">
+        <v>Tax treatment</v>
+      </c>
+      <c r="B13" s="20" t="str">
+        <v>Dropdown; blank = normal</v>
+      </c>
+      <c r="C13" s="20" t="str">
+        <v>Choose Normal tax calculation even when company pays tax. Exemption requires a genuine separate basis and evidence.</v>
+      </c>
+      <c r="D13" s="20" t="str">
+        <v>Normal tax calculation</v>
+      </c>
+    </row>
+    <row r="14" ht="76" customHeight="1">
+      <c r="A14" s="20" t="str">
+        <v>Exemption / tax basis</v>
+      </c>
+      <c r="B14" s="20" t="str">
+        <v>Only exemption/custom</v>
+      </c>
+      <c r="C14" s="20" t="str">
+        <v>Actual supporting basis and document; do not use net salary as the basis.</v>
+      </c>
+      <c r="D14" s="20" t="str">
+        <v>Leave blank for normal tax calculation</v>
+      </c>
+    </row>
+    <row r="15" ht="76" customHeight="1">
+      <c r="A15" s="20" t="str">
+        <v>Extra 1 name</v>
+      </c>
+      <c r="B15" s="20" t="str">
+        <v>Optional dropdown or custom</v>
+      </c>
+      <c r="C15" s="20" t="str">
+        <v>Name an additional approved component. Do not repeat existing allowances.</v>
+      </c>
+      <c r="D15" s="20" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="16" ht="76" customHeight="1">
+      <c r="A16" s="20" t="str">
+        <v>Extra 1 amount</v>
+      </c>
+      <c r="B16" s="20" t="str">
+        <v>When Extra name is filled</v>
+      </c>
+      <c r="C16" s="20" t="str">
+        <v>Approved component amount.</v>
+      </c>
+      <c r="D16" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="17" ht="76" customHeight="1">
+      <c r="A17" s="20" t="str">
+        <v>Extra 1 frequency</v>
+      </c>
+      <c r="B17" s="20" t="str">
+        <v>Dropdown</v>
+      </c>
+      <c r="C17" s="20" t="str">
+        <v>Recurring uses the package amount unit. One time requires a payable date.</v>
+      </c>
+      <c r="D17" s="20" t="str">
+        <v>Recurring</v>
+      </c>
+    </row>
+    <row r="18" ht="76" customHeight="1">
+      <c r="A18" s="20" t="str">
+        <v>Extra 1 payable date</v>
+      </c>
+      <c r="B18" s="20" t="str">
+        <v>One time only</v>
+      </c>
+      <c r="C18" s="20" t="str">
+        <v>Approved payment date. Leave blank for recurring.</v>
+      </c>
+      <c r="D18" s="20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="19" ht="76" customHeight="1">
+      <c r="A19" s="20" t="str">
+        <v>Extra 2 name</v>
+      </c>
+      <c r="B19" s="20" t="str">
+        <v>Optional dropdown or custom</v>
+      </c>
+      <c r="C19" s="20" t="str">
+        <v>Name an additional approved component. Do not repeat existing allowances.</v>
+      </c>
+      <c r="D19" s="20" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="20" ht="76" customHeight="1">
+      <c r="A20" s="20" t="str">
+        <v>Extra 2 amount</v>
+      </c>
+      <c r="B20" s="20" t="str">
+        <v>When Extra name is filled</v>
+      </c>
+      <c r="C20" s="20" t="str">
+        <v>Approved component amount.</v>
+      </c>
+      <c r="D20" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="21" ht="76" customHeight="1">
+      <c r="A21" s="20" t="str">
+        <v>Extra 2 frequency</v>
+      </c>
+      <c r="B21" s="20" t="str">
+        <v>Dropdown</v>
+      </c>
+      <c r="C21" s="20" t="str">
+        <v>Recurring uses the package amount unit. One time requires a payable date.</v>
+      </c>
+      <c r="D21" s="20" t="str">
+        <v>Recurring</v>
+      </c>
+    </row>
+    <row r="22" ht="76" customHeight="1">
+      <c r="A22" s="20" t="str">
+        <v>Extra 2 payable date</v>
+      </c>
+      <c r="B22" s="20" t="str">
+        <v>One time only</v>
+      </c>
+      <c r="C22" s="20" t="str">
+        <v>Approved payment date. Leave blank for recurring.</v>
+      </c>
+      <c r="D22" s="20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="23" ht="76" customHeight="1">
+      <c r="A23" s="20" t="str">
+        <v>Extra 3 name</v>
+      </c>
+      <c r="B23" s="20" t="str">
+        <v>Optional dropdown or custom</v>
+      </c>
+      <c r="C23" s="20" t="str">
+        <v>Name an additional approved component. Do not repeat existing allowances.</v>
+      </c>
+      <c r="D23" s="20" t="str">
+        <v>Meal allowance</v>
+      </c>
+    </row>
+    <row r="24" ht="76" customHeight="1">
+      <c r="A24" s="20" t="str">
+        <v>Extra 3 amount</v>
+      </c>
+      <c r="B24" s="20" t="str">
+        <v>When Extra name is filled</v>
+      </c>
+      <c r="C24" s="20" t="str">
+        <v>Approved component amount.</v>
+      </c>
+      <c r="D24" s="20" t="str">
+        <v>1000 (example only)</v>
+      </c>
+    </row>
+    <row r="25" ht="76" customHeight="1">
+      <c r="A25" s="20" t="str">
+        <v>Extra 3 frequency</v>
+      </c>
+      <c r="B25" s="20" t="str">
+        <v>Dropdown</v>
+      </c>
+      <c r="C25" s="20" t="str">
+        <v>Recurring uses the package amount unit. One time requires a payable date.</v>
+      </c>
+      <c r="D25" s="20" t="str">
+        <v>Recurring</v>
+      </c>
+    </row>
+    <row r="26" ht="76" customHeight="1">
+      <c r="A26" s="20" t="str">
+        <v>Extra 3 payable date</v>
+      </c>
+      <c r="B26" s="20" t="str">
+        <v>One time only</v>
+      </c>
+      <c r="C26" s="20" t="str">
+        <v>Approved payment date. Leave blank for recurring.</v>
+      </c>
+      <c r="D26" s="20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="27" ht="76" customHeight="1">
+      <c r="A27" s="20" t="str">
+        <v>Salary source</v>
+      </c>
+      <c r="B27" s="20" t="str">
+        <v>Required dropdown</v>
+      </c>
+      <c r="C27" s="20" t="str">
+        <v>Where approved salary comes from.</v>
+      </c>
+      <c r="D27" s="20" t="str">
+        <v>Current HRIS record</v>
+      </c>
+    </row>
+    <row r="28" ht="76" customHeight="1">
+      <c r="A28" s="20" t="str">
+        <v>PAN ID (if applicable)</v>
+      </c>
+      <c r="B28" s="20" t="str">
+        <v>Approved PAN only</v>
+      </c>
+      <c r="C28" s="20" t="str">
+        <v>Copy actual PAN record ID from HRIS; otherwise leave blank.</v>
+      </c>
+      <c r="D28" s="20" t="str">
+        <v>Leave blank for Current HRIS record</v>
+      </c>
+    </row>
+    <row r="29" ht="76" customHeight="1">
+      <c r="A29" s="20" t="str">
+        <v>Source document / note</v>
+      </c>
+      <c r="B29" s="20" t="str">
+        <v>Optional descriptive text</v>
+      </c>
+      <c r="C29" s="20" t="str">
+        <v>Actual source reference. Blank uses Salary source.</v>
+      </c>
+      <c r="D29" s="20" t="str">
+        <v>Current HRIS record checked on [date]</v>
+      </c>
+    </row>
+    <row r="30" ht="76" customHeight="1">
+      <c r="A30" s="20" t="str">
+        <v>Reason for this record</v>
+      </c>
+      <c r="B30" s="20" t="str">
+        <v>Required dropdown or text</v>
+      </c>
+      <c r="C30" s="20" t="str">
+        <v>Why this package is being recorded.</v>
+      </c>
+      <c r="D30" s="20" t="str">
+        <v>Initial setup</v>
+      </c>
+    </row>
+    <row r="31" ht="76" customHeight="1">
+      <c r="A31" s="20" t="str">
+        <v>Consultant agreement</v>
+      </c>
+      <c r="B31" s="20" t="str">
+        <v>Consultant row only</v>
+      </c>
+      <c r="C31" s="20" t="str">
+        <v>Actual distinct consulting engagement reference, not employee salary agreement.</v>
+      </c>
+      <c r="D31" s="20" t="str">
+        <v>Signed consulting agreement [reference/date]</v>
+      </c>
+    </row>
+    <row r="32" ht="76" customHeight="1">
+      <c r="A32" s="20" t="str">
+        <v>Consultant tax document</v>
+      </c>
+      <c r="B32" s="20" t="str">
+        <v>Consultant row only</v>
+      </c>
+      <c r="C32" s="20" t="str">
+        <v>Actual reviewed consultant withholding/tax-profile reference.</v>
+      </c>
+      <c r="D32" s="20" t="str">
+        <v>Finance-reviewed tax profile [reference]</v>
       </c>
     </row>
   </sheetData>

</xml_diff>